<commit_message>
chore(auto): daily pipeline 2026-05-20
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,19 +506,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mimo-v2-tts</t>
+          <t>Gemini 3.5 Flash</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -529,172 +529,176 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>语音</t>
+          <t>多模态</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/gemini-3.5-flash</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>基于自研Audio Tokenizer和多码本语音-文本联合建模架构；支持多粒度语音风格控制与单句内语气情感转折；支持多种方言及歌声合成</t>
+          <t>1048k上下文 [重要性:高|Google DeepMind 重点模型 Gemini 系列的重大版本更新子型号，具备较高行业关注度。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 官网→https://ai.google.dev/gemini-api/docs/models; 公司→Google DeepMind; 备注→多模态；Flash低延迟/高性价比子型号；约1M上下文; 问题: 官网字段为第三方排行榜 llm-stats.com，不是模型提供方官方页面; 模型发布时间为 2026-05-19，但当前信息来源为排行榜，建议核实 Google DeepMind / Google AI 官方公告; 公司名建议统一为 Google DeepMind; 模型名称包含具体系列、版本号与子型号，符合命名规范；未发现产品泛称问题，按 2026 年窗口内新模型保留。</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-13 11:52</t>
+          <t>2026-05-20 06:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mimo-v2.5-tts</t>
+          <t>Gemini 3.5 Pro</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>语音</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>multimodal large language model</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>采用“语言即控制”范式，支持自然语言指令控制语速、情绪与语气；包含标准版、VoiceDesign与VoiceClone三款模型，支持文本生成音色与高保真音色复刻；支持音频标签控制与分层导演剧本机制</t>
+          <t>Gemini 3.5系列中更强大的版本，具备更强推理与长程任务能力，当前处于内部测试阶段，后续将向更多用户分批发布。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:52</t>
-        </is>
-      </c>
+          <t>2026-05-20 06:02</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mimo-v2.5-tts-voiceclone</t>
+          <t>Gemini Omni</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>语音</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>video generation &amp; multimodal world model</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://mimo.xiaomi.com</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>仅需数秒参考音频即可高保真复刻真人音色，无需训练或微调；完整保留原说话人音色身份及气息、节奏、习惯性停顿等个性化特征；支持叠加自然语言指令、音频标签及导演剧本级脚本实现高自由度语音创作</t>
+          <t>基于世界模型技术的新型视频生成模型，支持文本/图像/音频/视频混合输入，可对话式编辑视频（如修改角色、背景、风格），并支持自拍驱动内容生成。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:52</t>
-        </is>
-      </c>
+          <t>2026-05-20 06:02</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mimo-v2.5-tts-voicedesign</t>
+          <t>文心大模型5.1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>百度</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -702,58 +706,54 @@
           <t>国内</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>语音</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>large language model</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>支持通过自然语言描述生成全新音色；支持多维度（年龄、性别、口音、音质、性格气质等）精细控制；无需参考音频即可从零构建声音形象</t>
+          <t>采用‘多维弹性预训练’技术，总参数压缩至前代约1/3、激活参数约1/2，预训练成本降至业界同规模模型约6%，聚焦效率与商业化落地。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:52</t>
-        </is>
-      </c>
+          <t>2026-05-20 06:02</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-opus-4.7-fast</t>
+          <t>GPT-5.5 Instant</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -761,109 +761,97 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>large language model</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://www.anthropic.com</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>支持3.75兆像素高分辨率图像输入；新增xhigh推理控制档位；引入任务预算机制优化智能体工作流；强化字面指令遵循能力</t>
+          <t>面向所有用户免费开放的轻量级GPT-5.5变体，主打简洁回答、强上下文记忆与快速响应，定位为高频日常交互主力模型。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:52</t>
-        </is>
-      </c>
+          <t>2026-05-20 06:02</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>perceptron-mk1</t>
+          <t>GLM-5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>智谱AI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>open-weight large language model</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>多模态模型；专注物理世界复杂动态处理；空间推理与视频理解能力强；API定价极低</t>
+          <t>744B参数开源大模型，于2026年2月发布，5月仍为当期全球开源模型性能标杆（Artificial Analysis榜单开源第一、综合第四），虽非5月19日首发，但在5月19日前后被密集报道并确认进入规模化商用部署阶段。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-02-XX</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:52</t>
-        </is>
-      </c>
+          <t>2026-05-20 06:02</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-21
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,352 +506,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash</t>
+          <t>文心大模型5.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>百度</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>多模态</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/gemini-3.5-flash</t>
-        </is>
-      </c>
+          <t>large language model</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1048k上下文 [重要性:高|Google DeepMind 重点模型 Gemini 系列的重大版本更新子型号，具备较高行业关注度。]</t>
+          <t>采用‘多维弹性预训练’技术，总参数压缩至前代约1/3、激活参数约1/2，预训练成本降至业界同规模模型约6%，聚焦效率与商业化落地。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-20 06:02</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>是</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 官网→https://ai.google.dev/gemini-api/docs/models; 公司→Google DeepMind; 备注→多模态；Flash低延迟/高性价比子型号；约1M上下文; 问题: 官网字段为第三方排行榜 llm-stats.com，不是模型提供方官方页面; 模型发布时间为 2026-05-19，但当前信息来源为排行榜，建议核实 Google DeepMind / Google AI 官方公告; 公司名建议统一为 Google DeepMind; 模型名称包含具体系列、版本号与子型号，符合命名规范；未发现产品泛称问题，按 2026 年窗口内新模型保留。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-20 06:01</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Gemini 3.5 Pro</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Google/DeepMind</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>multimodal large language model</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Gemini 3.5系列中更强大的版本，具备更强推理与长程任务能力，当前处于内部测试阶段，后续将向更多用户分批发布。</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-05-20 06:02</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Gemini Omni</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Google/DeepMind</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>video generation &amp; multimodal world model</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>基于世界模型技术的新型视频生成模型，支持文本/图像/音频/视频混合输入，可对话式编辑视频（如修改角色、背景、风格），并支持自拍驱动内容生成。</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-05-20 06:02</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>文心大模型5.1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>百度</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>large language model</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>采用‘多维弹性预训练’技术，总参数压缩至前代约1/3、激活参数约1/2，预训练成本降至业界同规模模型约6%，聚焦效率与商业化落地。</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-05-20 06:02</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>GPT-5.5 Instant</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>large language model</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>面向所有用户免费开放的轻量级GPT-5.5变体，主打简洁回答、强上下文记忆与快速响应，定位为高频日常交互主力模型。</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-05-20 06:02</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GLM-5</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>智谱AI</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>open-weight large language model</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>744B参数开源大模型，于2026年2月发布，5月仍为当期全球开源模型性能标杆（Artificial Analysis榜单开源第一、综合第四），虽非5月19日首发，但在5月19日前后被密集报道并确认进入规模化商用部署阶段。</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-02-XX</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-05-20 06:02</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
+          <t>2026-05-21 02:06</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-22
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,10 +530,14 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://yiyan.baidu.com</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>采用‘多维弹性预训练’技术，总参数压缩至前代约1/3、激活参数约1/2，预训练成本降至业界同规模模型约6%，聚焦效率与商业化落地。</t>
+          <t>采用‘多维弹性预训练’技术，总参数压缩至前代约1/3、激活参数约1/2，预训练成本降至业界同规模模型约6%，聚焦效率与商业化落地。 [重要性:中|百度属于国内优秀关注公司，文心大模型5.1若属官方版本更新则为值得关注的旗舰系列迭代。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -553,14 +557,179 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 任务类型→通用对话; 类型→基座模型; 公司→百度/文心; 备注→多维弹性预训练；参数与激活参数压缩；预训练成本显著降低；效率与商业化落地优化; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-09，位于追踪窗口前约12天，属于窗口前后1-2周内的新兴模型，应保留; 官网缺失，建议补充百度官方模型或文心/千帆官方页面; 尺寸/参数量缺失，且当前信息不足以可靠补全; 开闭源字段缺失，建议人工核实官方授权与开放方式; 现有发布时间与备注指向2026年新版本，但需以百度官方公告核实；不建议因采集时间早于窗口而删除。</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2026-05-22 02:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>非遗武术大模型 2.0</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>上海体育大学武术学院、百度飞桨智慧体育技术创新中心、上海体刻动视技术有限公司</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>垂直领域多模态视频分析大模型</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>面向非遗武术领域的AI视频分析智能平台，支持数秒级动作细节诊断、知识问答交互与专业报告生成。</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-05-22 02:09</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2026-05-21 02:06</t>
-        </is>
-      </c>
+      <c r="Q3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PuduFM 1.0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>普渡机器人</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>具身智能大模型</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>首个面向服务机器人的物理认知大模型，具备3D空间深度感知、物理状态预测与持续进化能力。</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-05-22 02:09</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>烽火工业智能体</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>中石化</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>行业垂直智能体</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>石油化工行业首个数字专家智能体，可直接操作工业软件、分析实时生产数据并运行工艺仿真。</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-05-22 02:09</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-23
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,7 +557,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 任务类型→通用对话; 类型→基座模型; 公司→百度/文心; 备注→多维弹性预训练；参数与激活参数压缩；预训练成本显著降低；效率与商业化落地优化; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-09，位于追踪窗口前约12天，属于窗口前后1-2周内的新兴模型，应保留; 官网缺失，建议补充百度官方模型或文心/千帆官方页面; 尺寸/参数量缺失，且当前信息不足以可靠补全; 开闭源字段缺失，建议人工核实官方授权与开放方式; 现有发布时间与备注指向2026年新版本，但需以百度官方公告核实；不建议因采集时间早于窗口而删除。</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 任务类型→通用对话; 类型→基座模型; 公司→百度/文心; 备注→多维弹性预训练；参数与激活参数压缩；预训练成本显著降低；效率与商业化落地优化; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-09，位于追踪窗口前约12天，属于窗口前后1-2周内的新兴模型，应保留; 官网缺失，建议补充百度官方模型或文心/千帆官方页面; 尺寸/参数量缺失，且当前信息不足以可靠补全; 开闭源字段缺失，建议人工核实官方授权与开放方式; 现有发布时间与备注指向2026年新版本，但需以百度官方公告核实；不建议因采集时间早于窗口而删除。; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 任务类型→通用对话; 类型→基座模型; 公司→百度/文心; 备注→多维弹性预训练；参数与激活参数压缩；预训练成本显著降低；效率与商业化落地优化; 开闭源→闭源; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-09，位于追踪窗口前约2周内，按宽松规则应保留; 官网为百度官方产品页，但建议进一步核实是否存在更精确的文心大模型/千帆官方模型页; 尺寸/参数量缺失，当前信息不足以可靠补全; 现有信息指向2026年新版本，但由于该时间点超出我的可靠知识范围，建议以百度官方公告复核发布日期与技术指标。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -596,7 +596,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>面向非遗武术领域的AI视频分析智能平台，支持数秒级动作细节诊断、知识问答交互与专业报告生成。</t>
+          <t>面向非遗武术领域的AI视频分析智能平台，支持数秒级动作细节诊断、知识问答交互与专业报告生成。 [重要性:低|高校与产业合作的垂直领域模型，应用场景明确但行业通用影响力有限。]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→视频分析/多模态理解; 类型→垂直领域多模态模型; 备注→非遗武术领域；动作细节诊断；知识问答；专业报告生成；视频分析; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-21，位于追踪窗口内，应保留; 官网缺失，建议补充模型提供方或项目官方发布页面; 公司主体较多，建议在数据库中统一为牵头单位或以联合发布形式规范记录; 尺寸/参数量缺失，当前信息不足以可靠补全; 开闭源情况缺失，建议人工核实; 该模型更像领域平台/多模态分析系统，需核实是否有独立模型权重、API或正式产品版本。</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -651,7 +651,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>首个面向服务机器人的物理认知大模型，具备3D空间深度感知、物理状态预测与持续进化能力。</t>
+          <t>首个面向服务机器人的物理认知大模型，具备3D空间深度感知、物理状态预测与持续进化能力。 [重要性:低|普渡机器人不在重点/优秀关注清单内，PuduFM 1.0属于具身智能垂直场景模型。]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→普渡机器人/Pudu Robotics; 国内外→国内; 任务类型→具身智能/机器人感知与规划; 类型→具身智能模型; 官网→https://www.pudurobotics.com; 备注→服务机器人；物理认知；3D空间感知；物理状态预测；持续学习; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-21，位于追踪窗口内，应保留; 原数据将普渡机器人标为国外不准确，普渡机器人为中国公司; 官网建议使用普渡机器人官方站点，若有PuduFM专页需进一步替换为模型专页; 尺寸/参数量缺失，当前信息不足以可靠补全; 开闭源情况缺失，建议人工核实; 具身智能方向值得观察，但当前信息不足以判断是否为通用基础模型还是面向自家机器人产品的内部能力。</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -726,10 +726,670 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称未体现明确版本号/型号，不符合本次模型名称规范; 原数据将中石化标为国外不准确，中石化为中国企业; 发布时间为2026-05-21，若属正式发布则位于窗口内，但因命名不合规仍建议不录入为模型条目; 官网缺失，建议补充中国石化或项目官方发布页面; 该条目更像行业智能体/应用系统，不一定是独立模型; 开闭源情况缺失，建议人工核实</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gemini Omni</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>多模态世界模型</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>具备物理一致性理解能力的世界模型，支持文本→三维视频生成与对话式视频编辑，首次实现动能、重力等物理属性的可推理建模。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>大语言模型（推理优化）</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>主打高性价比与超低延迟的Gemini新版本，在编码、Agent工具调用和响应速度（达其他前沿模型4倍tok/s）上显著超越Gemini 3.1 Pro。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Qwen 3.7-Max</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>通义千问旗舰新模型，Arena国产排名第一，支持35小时自主Agent内核运行，内核性能提升10倍，专为Agentic Cloud全栈调度优化。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>开源大语言模型</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Google最新开源轻量级模型，支持12GB显存下110 tok/s推理，强化数学与代码能力，与DeepSeek V4、Kimi K2.6等同期密集发布。</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DeepSeek V4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>深度求索/DeepSeek</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>开源大语言模型</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>深度求索新一代开源模型，聚焦长上下文与复杂推理，在多个开源基准测试中刷新SOTA，适配低成本边缘部署。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kimi K2.6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>月之暗面/Kimi</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Kimi系列最新闭源升级版，强化多文档RAG与垂类知识融合能力，面向金融、法律等专业场景提供增强型智能体接口。</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MiMo 2.5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>小米/MiMo</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>多模态端侧模型</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>小米自研轻量化多模态模型，支持手机端实时图文理解+语音指令闭环，集成于Xiaomi HyperOS 2.5 Agent框架。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GLM-5.1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>智谱AI/GLM</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>智谱GLM系列最新迭代，强化中文逻辑推理与安全对齐能力，原生支持GLM-Agent Runtime，已接入百炼平台。</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>代码智能体</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Anthropic正式发布的编程专用智能体，支持--json工作流、本地IDE深度集成及自动单元测试生成，日均迭代更新。</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gemini Spark</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>个人智能体</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>可在云端虚拟机全天候自主运行的个人AI智能体，支持跨应用任务编排、长期记忆与主动提醒，为Gemini生态首个量产级Agent产品。</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Antigravity 2.0</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>软件工程智能体平台</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>由93个子智能体协同构成的全自动代码生成平台，12小时内从零构建并测试完整操作系统，依托Gemini 3.5 Flash实现千美元级端到端成本。</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>锡望SeekWise大模型</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>无锡数字城市建设发展有限公司</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>垂类多模态智能体基座模型</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>全国首批通过信通院物联网智能体认证的AIoT大模型，聚焦钢材质检、锅炉优化、AGV接驳等实体产业场景，支持RAG+多智能体协同调度。</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-05-23 01:58</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-24
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>文心大模型5.1</t>
+          <t>Qwen 3.7-Max</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>百度</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -525,29 +525,25 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>large language model</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://yiyan.baidu.com</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>采用‘多维弹性预训练’技术，总参数压缩至前代约1/3、激活参数约1/2，预训练成本降至业界同规模模型约6%，聚焦效率与商业化落地。 [重要性:中|百度属于国内优秀关注公司，文心大模型5.1若属官方版本更新则为值得关注的旗舰系列迭代。]</t>
+          <t>通义千问旗舰新模型，Arena国产排名第一，支持35小时自主Agent内核运行，内核性能提升10倍，专为Agentic Cloud全栈调度优化。 [重要性:高|阿里/通义为国内重点关注公司，若为Max旗舰版本则属于重大模型更新。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-20 06:02</t>
+          <t>2026-05-23 01:58</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -557,38 +553,38 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 任务类型→通用对话; 类型→基座模型; 公司→百度/文心; 备注→多维弹性预训练；参数与激活参数压缩；预训练成本显著降低；效率与商业化落地优化; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-09，位于追踪窗口前约12天，属于窗口前后1-2周内的新兴模型，应保留; 官网缺失，建议补充百度官方模型或文心/千帆官方页面; 尺寸/参数量缺失，且当前信息不足以可靠补全; 开闭源字段缺失，建议人工核实官方授权与开放方式; 现有发布时间与备注指向2026年新版本，但需以百度官方公告核实；不建议因采集时间早于窗口而删除。; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 任务类型→通用对话; 类型→基座模型; 公司→百度/文心; 备注→多维弹性预训练；参数与激活参数压缩；预训练成本显著降低；效率与商业化落地优化; 开闭源→闭源; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-09，位于追踪窗口前约2周内，按宽松规则应保留; 官网为百度官方产品页，但建议进一步核实是否存在更精确的文心大模型/千帆官方模型页; 尺寸/参数量缺失，当前信息不足以可靠补全; 现有信息指向2026年新版本，但由于该时间点超出我的可靠知识范围，建议以百度官方公告复核发布日期与技术指标。</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→阿里巴巴/通义千问; 任务类型→通用对话; 官网→https://qwenlm.github.io; 备注→通义千问旗舰模型；Agentic能力；长程任务执行；面向云端智能体调度优化; 问题: 模型名称包含版本号，形式上符合规范; 截至已知公开资料无法核实“Qwen 3.7-Max”及其2026-05-20官方发布时间，建议人工复核官方公告; 原备注含有较多未经核实的榜单和性能表述，建议仅保留可官方验证的技术特征; 宽松保留；若无法找到阿里/通义官方发布页，应降级或删除。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-22 02:08</t>
+          <t>2026-05-24 02:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>非遗武术大模型 2.0</t>
+          <t>Gemma 4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>上海体育大学武术学院、百度飞桨智慧体育技术创新中心、上海体刻动视技术有限公司</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>垂直领域多模态视频分析大模型</t>
+          <t>开源大语言模型</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -596,17 +592,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>面向非遗武术领域的AI视频分析智能平台，支持数秒级动作细节诊断、知识问答交互与专业报告生成。 [重要性:低|高校与产业合作的垂直领域模型，应用场景明确但行业通用影响力有限。]</t>
+          <t>Google最新开源轻量级模型，支持12GB显存下110 tok/s推理，强化数学与代码能力，与DeepSeek V4、Kimi K2.6等同期密集发布。 [重要性:中|Gemma属于Google开放模型系列，重要性高于一般开源模型，但非Gemini旗舰线。]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-22 02:09</t>
+          <t>2026-05-23 01:58</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -616,52 +612,60 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→视频分析/多模态理解; 类型→垂直领域多模态模型; 备注→非遗武术领域；动作细节诊断；知识问答；专业报告生成；视频分析; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-21，位于追踪窗口内，应保留; 官网缺失，建议补充模型提供方或项目官方发布页面; 公司主体较多，建议在数据库中统一为牵头单位或以联合发布形式规范记录; 尺寸/参数量缺失，当前信息不足以可靠补全; 开闭源情况缺失，建议人工核实; 该模型更像领域平台/多模态分析系统，需核实是否有独立模型权重、API或正式产品版本。</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Google DeepMind; 任务类型→通用对话/代码生成; 官网→https://ai.google.dev/gemma; 备注→开放权重模型；轻量级部署；面向开发者本地与云端推理; 问题: 模型名称包含版本号，形式上符合规范; 截至已知公开资料无法核实“Gemma 4”及其2026-05-22官方发布时间，建议人工复核Google DeepMind或Google AI官方公告; 原备注中的“12GB显存下110 tok/s”等性能指标缺少可核实来源; 宽松保留；如确认为2026年Google官方发布的新一代Gemma，可继续录入。</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PuduFM 1.0</t>
+          <t>DeepSeek V4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>普渡机器人</t>
+          <t>深度求索/DeepSeek</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>具身智能大模型</t>
+          <t>开源大语言模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.deepseek.com/</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>首个面向服务机器人的物理认知大模型，具备3D空间深度感知、物理状态预测与持续进化能力。 [重要性:低|普渡机器人不在重点/优秀关注清单内，PuduFM 1.0属于具身智能垂直场景模型。]</t>
+          <t>深度求索新一代开源模型，聚焦长上下文与复杂推理，在多个开源基准测试中刷新SOTA，适配低成本边缘部署。 [重要性:高|DeepSeek新一代主力模型若属实，属于行业广泛关注的重大版本更新。]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-22 02:09</t>
+          <t>2026-05-23 01:58</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -671,52 +675,60 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→普渡机器人/Pudu Robotics; 国内外→国内; 任务类型→具身智能/机器人感知与规划; 类型→具身智能模型; 官网→https://www.pudurobotics.com; 备注→服务机器人；物理认知；3D空间感知；物理状态预测；持续学习; 问题: 模型名称包含明确版本号，符合规范; 发布时间为2026-05-21，位于追踪窗口内，应保留; 原数据将普渡机器人标为国外不准确，普渡机器人为中国公司; 官网建议使用普渡机器人官方站点，若有PuduFM专页需进一步替换为模型专页; 尺寸/参数量缺失，当前信息不足以可靠补全; 开闭源情况缺失，建议人工核实; 具身智能方向值得观察，但当前信息不足以判断是否为通用基础模型还是面向自家机器人产品的内部能力。</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 模型发布时间→2026-04-24; 公司→DeepSeek/深度求索; 任务类型→通用对话/复杂推理/代码生成; 官网→https://api-docs.deepseek.com; 备注→通用大语言模型；复杂推理；长上下文；低成本推理; 问题: 模型名称包含版本号，形式上符合规范; 原始发布时间2026-05-22疑似不是官方发布日期，需以官方公告日为准; 原备注中的“多个开源基准刷新SOTA”“边缘部署”等表述需官方或权威评测来源支撑; 按官方发布日期应修正为2026-04-24；虽在窗口前约一个月，但仍为2026年近期重大模型，建议保留并标注窗口外。</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>烽火工业智能体</t>
+          <t>MiMo 2.5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>中石化</t>
+          <t>小米/MiMo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>行业垂直智能体</t>
+          <t>多模态端侧模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://mimo.xiaomi.com</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>石油化工行业首个数字专家智能体，可直接操作工业软件、分析实时生产数据并运行工艺仿真。</t>
+          <t>小米自研轻量化多模态模型，支持手机端实时图文理解+语音指令闭环，集成于Xiaomi HyperOS 2.5 Agent框架。 [重要性:中|小米/MiMo属于国内优秀关注公司，端侧多模态模型具备特定场景价值。]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-22 02:09</t>
+          <t>2026-05-23 01:58</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -726,22 +738,26 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称未体现明确版本号/型号，不符合本次模型名称规范; 原数据将中石化标为国外不准确，中石化为中国企业; 发布时间为2026-05-21，若属正式发布则位于窗口内，但因命名不合规仍建议不录入为模型条目; 官网缺失，建议补充中国石化或项目官方发布页面; 该条目更像行业智能体/应用系统，不一定是独立模型; 开闭源情况缺失，建议人工核实</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→小米/MiMo; 任务类型→端侧多模态/图文理解/语音交互; 备注→端侧多模态模型；移动设备部署；图文理解；语音指令交互; 问题: 模型名称包含版本号，形式上符合规范; 截至已知公开资料无法核实“MiMo 2.5”及其2026-05-22官方发布时间，建议人工复核小米官方技术公告; 原备注中“HyperOS 2.5 Agent框架”等产品集成信息需确认是否为模型自身特征; 宽松保留；若仅为系统功能或Agent框架而非模型版本，应调整分类。</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gemini Omni</t>
+          <t>Claude Code</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -753,20 +769,24 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>多模态世界模型</t>
+          <t>代码智能体</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://docs.anthropic.com/en/docs/claude-code/overview</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>具备物理一致性理解能力的世界模型，支持文本→三维视频生成与对话式视频编辑，首次实现动能、重力等物理属性的可推理建模。</t>
+          <t>Anthropic正式发布的编程专用智能体，支持--json工作流、本地IDE深度集成及自动单元测试生成，日均迭代更新。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -781,15 +801,19 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 不是具体模型名称，属于Anthropic的代码智能体产品/工具; 发布时间应为2025年相关发布/GA时间，属于旧产品（发布于2025年）; 原始模型发布时间2026-05-22疑似错误</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash</t>
+          <t>Gemini Spark</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -808,7 +832,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>大语言模型（推理优化）</t>
+          <t>个人智能体</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -816,7 +840,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>主打高性价比与超低延迟的Gemini新版本，在编码、Agent工具调用和响应速度（达其他前沿模型4倍tok/s）上显著超越Gemini 3.1 Pro。</t>
+          <t>可在云端虚拟机全天候自主运行的个人AI智能体，支持跨应用任务编排、长期记忆与主动提醒，为Gemini生态首个量产级Agent产品。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -836,34 +860,38 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(低置信)待人工确认 — 建议删除：产品泛称无版本号; 缺少明确版本号/型号，不符合“具体模型/产品名称 + 版本号/型号”的命名要求; 更像个人智能体产品而非具体模型; 截至已知公开资料无法核实“Gemini Spark”及其2026-05-21官方发布时间</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Qwen 3.7-Max</t>
+          <t>Antigravity 2.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>软件工程智能体平台</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -871,12 +899,12 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>通义千问旗舰新模型，Arena国产排名第一，支持35小时自主Agent内核运行，内核性能提升10倍，专为Agentic Cloud全栈调度优化。</t>
+          <t>由93个子智能体协同构成的全自动代码生成平台，12小时内从零构建并测试完整操作系统，依托Gemini 3.5 Flash实现千美元级端到端成本。 [重要性:中|Google DeepMind相关软件工程智能体平台值得关注，但不是Gemini旗舰模型本身。]</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -891,22 +919,26 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Google DeepMind; 任务类型→软件工程智能体/代码生成; 类型→软件工程智能体平台; 备注→软件工程智能体平台；多智能体协作；代码生成；自动测试；端到端软件构建; 问题: 名称包含版本号，形式上符合规范; 该条目更像智能体平台/开发工具，而非具体基础模型; 截至已知公开资料无法核实“Antigravity 2.0”及其2026-05-21官方发布时间; 原备注中“93个子智能体”“12小时构建完整操作系统”“千美元级成本”等表述高度具体但缺少可核实来源; 宽松保留为智能体平台条目；若数据库只收录模型，应改为记录其实际底座模型，例如Gemini的具体版本。</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gemma 4</t>
+          <t>锡望SeekWise大模型</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>无锡数字城市建设发展有限公司</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -918,20 +950,24 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>开源大语言模型</t>
+          <t>垂类多模态智能体基座模型</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://seekvision.cn</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Google最新开源轻量级模型，支持12GB显存下110 tok/s推理，强化数学与代码能力，与DeepSeek V4、Kimi K2.6等同期密集发布。</t>
+          <t>全国首批通过信通院物联网智能体认证的AIoT大模型，聚焦钢材质检、锅炉优化、AGV接驳等实体产业场景，支持RAG+多智能体协同调度。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -946,22 +982,26 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(低置信)待人工确认 — 建议删除：缺少版本号/型号; 名称不是“具体模型/产品名称 + 版本号/型号”的规范形式; 国内外字段错误：无锡数字城市建设发展有限公司为中国公司，应标注为国内; “垂类多模态智能体基座模型”分类表述混杂，建议改为行业模型或工业AIoT智能体; 截至已知公开资料无法核实其2026-05-21官方发布时间</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:04</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DeepSeek V4</t>
+          <t>GLM-5.1-HighSpeed</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>深度求索/DeepSeek</t>
+          <t>智谱AI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -973,7 +1013,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>开源大语言模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -981,17 +1021,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>深度求索新一代开源模型，聚焦长上下文与复杂推理，在多个开源基准测试中刷新SOTA，适配低成本边缘部署。</t>
+          <t>官方称推理速度达400 tokens/s，面向高吞吐低延迟场景优化的GLM系列新版本</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-24 02:07</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1009,26 +1049,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kimi K2.6</t>
+          <t>BitCPM-CANN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>月之暗面/Kimi</t>
+          <t>OpenBMB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>大语言模型（昇腾原生）</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1036,17 +1076,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Kimi系列最新闭源升级版，强化多文档RAG与垂类知识融合能力，面向金融、法律等专业场景提供增强型智能体接口。</t>
+          <t>基于华为昇腾910B芯片全栈原生训练的开源大模型，适配CANN生态，强调国产算力高效部署</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-24 02:07</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1064,14 +1104,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MiMo 2.5</t>
+          <t>Confucius4-TTS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>小米/MiMo</t>
+          <t>网易有道</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1083,7 +1123,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>多模态端侧模型</t>
+          <t>语音合成模型</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1091,17 +1131,17 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>小米自研轻量化多模态模型，支持手机端实时图文理解+语音指令闭环，集成于Xiaomi HyperOS 2.5 Agent框架。</t>
+          <t>支持14种语言零样本语音克隆的TTS引擎，即将全量开源</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-24 02:07</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1119,26 +1159,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GLM-5.1</t>
+          <t>AlphaProof Nexus</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>智谱AI/GLM</t>
+          <t>Google DeepMind</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>数学推理与形式化证明框架</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1146,17 +1186,17 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>智谱GLM系列最新迭代，强化中文逻辑推理与安全对齐能力，原生支持GLM-Agent Runtime，已接入百炼平台。</t>
+          <t>首个端到端可验证数学证明生成系统，集成强化学习驱动的搜索与Coq/Galaxy形式化验证闭环</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-24 02:07</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1174,7 +1214,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Claude Code</t>
+          <t>Mythos Preview</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1193,7 +1233,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>代码智能体</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1201,7 +1241,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Anthropic正式发布的编程专用智能体，支持--json工作流、本地IDE深度集成及自动单元测试生成，日均迭代更新。</t>
+          <t>Anthropic发布的‘史上最强’预览版大模型，因安全评估风险被宣布无限期封印，仅限Glasswing漏洞挖掘计划内部使用</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1211,7 +1251,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-24 02:07</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1225,171 +1265,6 @@
         </is>
       </c>
       <c r="Q14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Gemini Spark</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Google/DeepMind</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>个人智能体</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>可在云端虚拟机全天候自主运行的个人AI智能体，支持跨应用任务编排、长期记忆与主动提醒，为Gemini生态首个量产级Agent产品。</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2026-05-23 01:58</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Antigravity 2.0</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Google/DeepMind</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>软件工程智能体平台</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>由93个子智能体协同构成的全自动代码生成平台，12小时内从零构建并测试完整操作系统，依托Gemini 3.5 Flash实现千美元级端到端成本。</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>2026-05-23 01:58</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>锡望SeekWise大模型</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>无锡数字城市建设发展有限公司</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>垂类多模态智能体基座模型</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>全国首批通过信通院物联网智能体认证的AIoT大模型，聚焦钢材质检、锅炉优化、AGV接驳等实体产业场景，支持RAG+多智能体协同调度。</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>2026-05-23 01:58</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-25
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,73 +506,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Qwen 3.7-Max</t>
+          <t>gamma-world-test</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>大语言模型</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/gamma-world-test</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>通义千问旗舰新模型，Arena国产排名第一，支持35小时自主Agent内核运行，内核性能提升10倍，专为Agentic Cloud全栈调度优化。 [重要性:高|阿里/通义为国内重点关注公司，若为Max旗舰版本则属于重大模型更新。]</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→阿里巴巴/通义千问; 任务类型→通用对话; 官网→https://qwenlm.github.io; 备注→通义千问旗舰模型；Agentic能力；长程任务执行；面向云端智能体调度优化; 问题: 模型名称包含版本号，形式上符合规范; 截至已知公开资料无法核实“Qwen 3.7-Max”及其2026-05-20官方发布时间，建议人工复核官方公告; 原备注含有较多未经核实的榜单和性能表述，建议仅保留可官方验证的技术特征; 宽松保留；若无法找到阿里/通义官方发布页，应降级或删除。</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gamma-world-test)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-24 02:04</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gemma 4</t>
+          <t>Fun-ASR-Nano-2512-hf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>阿里</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,92 +588,96 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>开源大语言模型</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>语音</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/FunAudioLLM/Fun-ASR-Nano-2512-hf</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Google最新开源轻量级模型，支持12GB显存下110 tok/s推理，强化数学与代码能力，与DeepSeek V4、Kimi K2.6等同期密集发布。 [重要性:中|Gemma属于Google开放模型系列，重要性高于一般开源模型，但非Gemini旗舰线。]</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Google DeepMind; 任务类型→通用对话/代码生成; 官网→https://ai.google.dev/gemma; 备注→开放权重模型；轻量级部署；面向开发者本地与云端推理; 问题: 模型名称包含版本号，形式上符合规范; 截至已知公开资料无法核实“Gemma 4”及其2026-05-22官方发布时间，建议人工复核Google DeepMind或Google AI官方公告; 原备注中的“12GB显存下110 tok/s”等性能指标缺少可核实来源; 宽松保留；如确认为2026年Google官方发布的新一代Gemma，可继续录入。</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Fun-ASR-Nano-2512-hf)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-24 02:04</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DeepSeek V4</t>
+          <t>Gemini 3.5 Flash</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>深度求索/DeepSeek</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>开源大语言模型</t>
+          <t>multimodal large language model</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://www.deepseek.com/</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>深度求索新一代开源模型，聚焦长上下文与复杂推理，在多个开源基准测试中刷新SOTA，适配低成本边缘部署。 [重要性:高|DeepSeek新一代主力模型若属实，属于行业广泛关注的重大版本更新。]</t>
+          <t>Google I/O 2026 发布的轻量级高性能模型，主打极低延迟、高吞吐（每秒Token数为前沿模型4倍）与强Agent工具调用能力，当日上线可用。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -675,60 +687,52 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 模型发布时间→2026-04-24; 公司→DeepSeek/深度求索; 任务类型→通用对话/复杂推理/代码生成; 官网→https://api-docs.deepseek.com; 备注→通用大语言模型；复杂推理；长上下文；低成本推理; 问题: 模型名称包含版本号，形式上符合规范; 原始发布时间2026-05-22疑似不是官方发布日期，需以官方公告日为准; 原备注中的“多个开源基准刷新SOTA”“边缘部署”等表述需官方或权威评测来源支撑; 按官方发布日期应修正为2026-04-24；虽在窗口前约一个月，但仍为2026年近期重大模型，建议保留并标注窗口外。</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:04</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MiMo 2.5</t>
+          <t>Gemini Omni</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>小米/MiMo</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>多模态端侧模型</t>
+          <t>world model / physics-aware multimodal model</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://mimo.xiaomi.com</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>小米自研轻量化多模态模型，支持手机端实时图文理解+语音指令闭环，集成于Xiaomi HyperOS 2.5 Agent框架。 [重要性:中|小米/MiMo属于国内优秀关注公司，端侧多模态模型具备特定场景价值。]</t>
+          <t>具备物理一致性理解能力的世界模型，支持跨文本-视频的三维空间建模、动能/重力模拟及对话式视频元素编辑。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -738,60 +742,52 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→小米/MiMo; 任务类型→端侧多模态/图文理解/语音交互; 备注→端侧多模态模型；移动设备部署；图文理解；语音指令交互; 问题: 模型名称包含版本号，形式上符合规范; 截至已知公开资料无法核实“MiMo 2.5”及其2026-05-22官方发布时间，建议人工复核小米官方技术公告; 原备注中“HyperOS 2.5 Agent框架”等产品集成信息需确认是否为模型自身特征; 宽松保留；若仅为系统功能或Agent框架而非模型版本，应调整分类。</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:04</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Claude Code</t>
+          <t>文心大模型5.1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>百度</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>代码智能体</t>
+          <t>large language model</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://docs.anthropic.com/en/docs/claude-code/overview</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Anthropic正式发布的编程专用智能体，支持--json工作流、本地IDE深度集成及自动单元测试生成，日均迭代更新。</t>
+          <t>采用‘多维弹性预训练’技术，预训练成本降至同规模模型约6%，总参数压缩至1/3，激活参数压缩至1/2，聚焦长程智能体与效率优化。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -801,26 +797,22 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 不是具体模型名称，属于Anthropic的代码智能体产品/工具; 发布时间应为2025年相关发布/GA时间，属于旧产品（发布于2025年）; 原始模型发布时间2026-05-22疑似错误</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:04</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gemini Spark</t>
+          <t>GPT-5.5 Instant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -832,7 +824,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>个人智能体</t>
+          <t>large language model</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -840,17 +832,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>可在云端虚拟机全天候自主运行的个人AI智能体，支持跨应用任务编排、长期记忆与主动提醒，为Gemini生态首个量产级Agent产品。</t>
+          <t>面向全体用户免费开放的轻量化GPT-5迭代版，强调简洁响应、增强长期记忆能力与低开销推理，标志OpenAI向价值验证与普惠部署转向。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -860,26 +852,22 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(低置信)待人工确认 — 建议删除：产品泛称无版本号; 缺少明确版本号/型号，不符合“具体模型/产品名称 + 版本号/型号”的命名要求; 更像个人智能体产品而非具体模型; 截至已知公开资料无法核实“Gemini Spark”及其2026-05-21官方发布时间</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:04</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Antigravity 2.0</t>
+          <t>Claude Opus 4.7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -891,7 +879,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>软件工程智能体平台</t>
+          <t>large language model</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -899,17 +887,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>由93个子智能体协同构成的全自动代码生成平台，12小时内从零构建并测试完整操作系统，依托Gemini 3.5 Flash实现千美元级端到端成本。 [重要性:中|Google DeepMind相关软件工程智能体平台值得关注，但不是Gemini旗舰模型本身。]</t>
+          <t>虽发布于4月，但其争议性表现（幻觉加剧、任务偷懒）在5月24日前持续发酵并被主流媒体集中报道，被行业视为‘倒退型更新’典型，故纳入5月关键模型事件。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-04-XX</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -919,26 +907,22 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Google DeepMind; 任务类型→软件工程智能体/代码生成; 类型→软件工程智能体平台; 备注→软件工程智能体平台；多智能体协作；代码生成；自动测试；端到端软件构建; 问题: 名称包含版本号，形式上符合规范; 该条目更像智能体平台/开发工具，而非具体基础模型; 截至已知公开资料无法核实“Antigravity 2.0”及其2026-05-21官方发布时间; 原备注中“93个子智能体”“12小时构建完整操作系统”“千美元级成本”等表述高度具体但缺少可核实来源; 宽松保留为智能体平台条目；若数据库只收录模型，应改为记录其实际底座模型，例如Gemini的具体版本。</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:04</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>锡望SeekWise大模型</t>
+          <t>Antigravity 2.0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>无锡数字城市建设发展有限公司</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -950,29 +934,25 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>垂类多模态智能体基座模型</t>
+          <t>autonomous agent platform</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>https://seekvision.cn</t>
-        </is>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>全国首批通过信通院物联网智能体认证的AIoT大模型，聚焦钢材质检、锅炉优化、AGV接驳等实体产业场景，支持RAG+多智能体协同调度。</t>
+          <t>基于多智能体协同的全自动代码生成平台，支持93个子智能体并行工作，12小时内从零构建含调度、内存管理、文件系统的完整操作系统。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-23 01:58</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -982,38 +962,34 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(低置信)待人工确认 — 建议删除：缺少版本号/型号; 名称不是“具体模型/产品名称 + 版本号/型号”的规范形式; 国内外字段错误：无锡数字城市建设发展有限公司为中国公司，应标注为国内; “垂类多模态智能体基座模型”分类表述混杂，建议改为行业模型或工业AIoT智能体; 截至已知公开资料无法核实其2026-05-21官方发布时间</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:04</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GLM-5.1-HighSpeed</t>
+          <t>Gemini Spark</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>智谱AI</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>personal autonomous agent</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1021,17 +997,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>官方称推理速度达400 tokens/s，面向高吞吐低延迟场景优化的GLM系列新版本</t>
+          <t>首个可在云端虚拟机中全天候自主运行的个人智能体，专为软件工程自动化设计，支持长期状态维持与跨会话任务延续。</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-24 02:07</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1049,26 +1025,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BitCPM-CANN</t>
+          <t>昇腾AgentInfra</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OpenBMB</t>
+          <t>华为</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>大语言模型（昇腾原生）</t>
+          <t>agent runtime infrastructure</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1076,17 +1052,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>基于华为昇腾910B芯片全栈原生训练的开源大模型，适配CANN生态，强调国产算力高效部署</t>
+          <t>华为鲲鹏昇腾开发者大会上发布的智能体原生运行环境，作为‘鲲鹏硬核算力 + openEuler异构系统 + AgentInfra’三层架构核心组件全面开源。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-24 02:07</t>
+          <t>2026-05-25 02:13</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1100,171 +1076,6 @@
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Confucius4-TTS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>网易有道</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>语音合成模型</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>支持14种语言零样本语音克隆的TTS引擎，即将全量开源</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:07</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AlphaProof Nexus</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Google DeepMind</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>数学推理与形式化证明框架</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>首个端到端可验证数学证明生成系统，集成强化学习驱动的搜索与Coq/Galaxy形式化验证闭环</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:07</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Mythos Preview</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>大语言模型</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Anthropic发布的‘史上最强’预览版大模型，因安全评估风险被宣布无限期封印，仅限Glasswing漏洞挖掘计划内部使用</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>2026-05-24 02:07</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-27
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,61 +506,435 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>昇腾AgentInfra</t>
+          <t>vermeer-XL-CA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>华为</t>
+          <t>微软</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>agent runtime infrastructure</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/microsoft/vermeer-XL-CA</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>华为鲲鹏昇腾开发者大会上发布的智能体原生运行环境，作为‘鲲鹏硬核算力 + openEuler异构系统 + AgentInfra’三层架构核心组件全面开源。</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-25 02:13</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-XL-CA)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>vermeer-XL</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>微软</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/microsoft/vermeer-XL</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-XL)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>vermeer-L-AP</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>微软</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/microsoft/vermeer-L-AP</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-L-AP)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>vermeer-L</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>微软</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/microsoft/vermeer-L</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-L)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Grok V9-Medium</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SpaceXAI (xAI)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1.5T参数基础模型，已完成训练并进入微调阶段，专为复杂编程任务优化，预计2–3周内公开发布，年底将开源0.5T版本。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 非具体模型条目：昇腾AgentInfra更像智能体运行环境/基础设施组件，不属于模型名称; 模型名称缺少明确版本号或型号; 类型分类不应归为模型，应归为智能体基础设施/运行时</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2026-05-26 02:03</t>
-        </is>
-      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MiniCPM5-1B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>OpenBMB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>小规模混合推理大语言模型</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>10.8亿参数开源模型，登顶Artificial Analysis小模型榜单（17.9分），支持INT4量化（约0.5GB），可在手机、浏览器及CPU本地运行。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash (Low)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Google / DeepMind</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>轻量级多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Antigravity平台新增的低延迟、低成本推理变体，面向高并发轻负载场景优化，为Gemini 3.5系列首次推出的‘Flash’分级型号。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-28
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vermeer-XL-CA</t>
+          <t>Grok V9-Medium</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>SpaceXAI (xAI)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,31 +521,19 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/microsoft/vermeer-XL-CA</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>1.5T参数基础模型，已完成训练并进入微调阶段，专为复杂编程任务优化，预计2–3周内公开发布，年底将开源0.5T版本。 [重要性:中|xAI 属于国外优秀关注公司，若该模型属实则为 Grok 系列较重要的新版本/子变体。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -555,32 +543,36 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+          <t>2026-05-27 02:12</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-XL-CA)</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→xAI; 官网→https://docs.x.ai/docs/models; 任务类型→通用对话/代码生成; 问题: 公司名不规范：'SpaceXAI (xAI)' 应统一为 'xAI'，xAI 与 SpaceX 是不同主体; 模型名称形式上符合规范：包含具体产品名与版本/型号，不属于产品泛称; 模型存在性与官方发布时间需人工核实：截至可确认信息范围内，未能确认 xAI 官方发布过 'Grok V9-Medium'; 当前备注包含较多预测性/传闻信息，如'进入微调阶段'、'预计2–3周内公开发布'、'年底将开源0.5T版本'，建议核验官方来源后再录入; 模型发布时间 2026-05-26 与追踪窗口相近，但需确认是否为 xAI 官方发布日期，而非传闻日期或采集日期; 不建议因无法核实而直接删除；按规则仅产品泛称或2025年及以前旧模型应删除。建议后续以 xAI 官网、官方博客或官方 X 账号公告为准复核。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-27 02:12</t>
+          <t>2026-05-28 01:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>vermeer-XL</t>
+          <t>Assemble_Trocar</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -607,7 +599,7 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/vermeer-XL</t>
+          <t>https://huggingface.co/nvidia/Assemble_Trocar</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -617,37 +609,37 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-XL)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Assemble_Trocar)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-27 02:12</t>
+          <t>2026-05-28 01:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>vermeer-L-AP</t>
+          <t>GPT-5.6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -655,66 +647,54 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/microsoft/vermeer-L-AP</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>泄露信息显示支持150万token超长上下文窗口，预计2026年6月正式发布</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
+          <t>2026-05-28 01:56</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-L-AP)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-05-27 02:12</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>vermeer-L</t>
+          <t>Claude Mythos</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -722,66 +702,54 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>大语言模型（安全增强型）</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/microsoft/vermeer-L</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>在欧洲央行委托的红队测试中意外暴露SWIFT及三大央行结算系统漏洞，属Mythos系列新安全推理模型</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
+          <t>2026-05-28 01:56</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/vermeer-L)</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-05-27 02:12</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Grok V9-Medium</t>
+          <t>Gemini for Science</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SpaceXAI (xAI)</t>
+          <t>Google DeepMind / Google Research</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -793,7 +761,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>多模态科学大模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -801,17 +769,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1.5T参数基础模型，已完成训练并进入微调阶段，专为复杂编程任务优化，预计2–3周内公开发布，年底将开源0.5T版本。</t>
+          <t>面向生命科学与实验推理的专用Gemini变体，集成Science Skills工具链，支持假设生成、实验设计与论文级文献推理</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-27 02:12</t>
+          <t>2026-05-28 01:56</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -829,14 +797,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MiniCPM5-1B</t>
+          <t>Protenix-v2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OpenBMB</t>
+          <t>未知（据信为中美联合生物AI初创团队）</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -848,7 +816,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>小规模混合推理大语言模型</t>
+          <t>蛋白质结构与功能预测模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -856,17 +824,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>10.8亿参数开源模型，登顶Artificial Analysis小模型榜单（17.9分），支持INT4量化（约0.5GB），可在手机、浏览器及CPU本地运行。</t>
+          <t>开源蛋白质语言模型v2版本，支持端到端突变效应预测与条件性折叠生成，在CAMEO基准上刷新SOTA</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-27 02:12</t>
+          <t>2026-05-28 01:56</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -884,14 +852,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash (Low)</t>
+          <t>WholebodyVLA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Google / DeepMind</t>
+          <t>Google Research</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -903,7 +871,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>轻量级多模态大语言模型</t>
+          <t>具身多模态智能体（VLA）</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -911,30 +879,85 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Antigravity平台新增的低延迟、低成本推理变体，面向高并发轻负载场景优化，为Gemini 3.5系列首次推出的‘Flash’分级型号。</t>
+          <t>首个覆盖全身运动控制（含手指微操、步态平衡、双臂协同）的视觉-语言-动作联合模型，专为通用机器人任务设计</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-05-28 01:56</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AI决策机器人R1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NBBOSS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>商业决策智能体</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>首款面向企业高管的可分离式AI决策智能体，融合实时BI数据接入、因果推断引擎与会议纪要自动生成模块</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-05-27 02:12</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-05-28 01:56</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-29
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Grok V9-Medium</t>
+          <t>GPT-5.6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SpaceXAI (xAI)</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -533,17 +533,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1.5T参数基础模型，已完成训练并进入微调阶段，专为复杂编程任务优化，预计2–3周内公开发布，年底将开源0.5T版本。 [重要性:中|xAI 属于国外优秀关注公司，若该模型属实则为 Grok 系列较重要的新版本/子变体。]</t>
+          <t>泄露信息显示支持150万token超长上下文窗口，预计2026年6月正式发布 [重要性:高|OpenAI 的 GPT 主线模型若属实将是旗舰级重大版本更新。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-27 02:12</t>
+          <t>2026-05-28 01:56</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -553,26 +553,26 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→xAI; 官网→https://docs.x.ai/docs/models; 任务类型→通用对话/代码生成; 问题: 公司名不规范：'SpaceXAI (xAI)' 应统一为 'xAI'，xAI 与 SpaceX 是不同主体; 模型名称形式上符合规范：包含具体产品名与版本/型号，不属于产品泛称; 模型存在性与官方发布时间需人工核实：截至可确认信息范围内，未能确认 xAI 官方发布过 'Grok V9-Medium'; 当前备注包含较多预测性/传闻信息，如'进入微调阶段'、'预计2–3周内公开发布'、'年底将开源0.5T版本'，建议核验官方来源后再录入; 模型发布时间 2026-05-26 与追踪窗口相近，但需确认是否为 xAI 官方发布日期，而非传闻日期或采集日期; 不建议因无法核实而直接删除；按规则仅产品泛称或2025年及以前旧模型应删除。建议后续以 xAI 官网、官方博客或官方 X 账号公告为准复核。</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://platform.openai.com/docs/models; 任务类型→通用对话; 开闭源→闭源; 问题: 未能确认 OpenAI 官方发布过 GPT-5.6; 现有发布时间疑似来自泄露或传闻，不应视为官方发布日期; 备注包含预测和泄露信息，建议人工核验后再录入; 模型名称包含明确版本号，形式上符合规范；但发布真实性和官方发布日期需重点复核。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-28 01:55</t>
+          <t>2026-05-29 02:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Assemble_Trocar</t>
+          <t>Claude Mythos</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,31 +580,19 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>大语言模型（安全增强型）</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/Assemble_Trocar</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>在欧洲央行委托的红队测试中意外暴露SWIFT及三大央行结算系统漏洞，属Mythos系列新安全推理模型</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -614,32 +602,36 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>2026-05-28 01:56</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Assemble_Trocar)</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称像系列名或代号，未指向具体模型版本; 未能确认 Anthropic 官方发布过 Claude Mythos; 备注中关于央行和 SWIFT 漏洞暴露的描述高度异常，需严格核验来源; 现有发布时间缺乏官方依据</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-28 01:55</t>
+          <t>2026-05-29 02:03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GPT-5.6</t>
+          <t>Claude Opus 4.8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -647,66 +639,86 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>大语言模型</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/claude-opus-4-8</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>泄露信息显示支持150万token超长上下文窗口，预计2026年6月正式发布</t>
+          <t>1000k上下文；顶级推理能力；顶级编码能力；高端定价 [重要性:高|Anthropic Claude Opus 主线高端模型若属实属于旗舰级重大版本更新。]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>New</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+          <t>llm-stats.com 排行榜; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://docs.anthropic.com/en/docs/about-claude/models/overview; 公司→Anthropic; 开闭源→闭源; 问题: 官网字段为第三方排行榜链接，不是 Anthropic 官方页面; 未能确认 Anthropic 官方发布过 Claude Opus 4.8; 模型发布时间需以 Anthropic 官方公告或官方模型文档为准; llm-stats.com 排行榜不应作为官方发布依据; 模型名称包含系列、档位和版本号，形式上符合规范；但该条目的发布时间、上下文长度和能力描述均需官方核验。</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-05-29 02:03</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Claude Mythos</t>
+          <t>Qwen3.7-Max</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>大语言模型（安全增强型）</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -714,17 +726,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>在欧洲央行委托的红队测试中意外暴露SWIFT及三大央行结算系统漏洞，属Mythos系列新安全推理模型</t>
+          <t>阿里云于2026年5月20日阿里云峰会发布的面向AI Agent场景设计的新旗舰模型，在编程、推理、工具调用等能力上显著强化，支持长时间运行与多次工具调用，在Code Arena榜单中得分1541。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
+          <t>2026-05-29 02:04</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -742,26 +754,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gemini for Science</t>
+          <t>DeepSeek-V4 Flash</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Google DeepMind / Google Research</t>
+          <t>深度求索/DeepSeek</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>多模态科学大模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -769,17 +781,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>面向生命科学与实验推理的专用Gemini变体，集成Science Skills工具链，支持假设生成、实验设计与论文级文献推理</t>
+          <t>DeepSeek于2026年5月28日最新发布的高性价比推理优化版本，提供$0.14/M token定价及每日200万Token免费额度，主打高并发、低成本商用场景。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
+          <t>2026-05-29 02:04</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -797,26 +809,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Protenix-v2</t>
+          <t>豆包Seed 2.0 Pro</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>未知（据信为中美联合生物AI初创团队）</t>
+          <t>字节跳动/豆包</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>蛋白质结构与功能预测模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -824,17 +836,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>开源蛋白质语言模型v2版本，支持端到端突变效应预测与条件性折叠生成，在CAMEO基准上刷新SOTA</t>
+          <t>豆包于2026年5月28日前后正式发布升级版Seed 2.0 Pro，综合性能跻身全球前五，以$1/M token超低价格和MMMU-Pro 68.7%精度成为国产综合能力最强的商用大模型之一。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
+          <t>2026-05-29 02:04</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -852,14 +864,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WholebodyVLA</t>
+          <t>HappyHorse 1.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Google Research</t>
+          <t>HappyHorse</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -871,7 +883,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>具身多模态智能体（VLA）</t>
+          <t>视频生成模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -879,17 +891,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>首个覆盖全身运动控制（含手指微操、步态平衡、双臂协同）的视觉-语言-动作联合模型，专为通用机器人任务设计</t>
+          <t>2026年5月28日官宣发布的首个专注高质量长时序视频生成的多模态基础模型，被列为2026年5月AI模型排行榜‘视频生成’唯一代表，以SOTA视频质量定位内容创作者市场。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
+          <t>2026-05-29 02:04</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -907,14 +919,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AI决策机器人R1</t>
+          <t>Meta One Plus / Meta One Premium</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NBBOSS</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -926,7 +938,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>商业决策智能体</t>
+          <t>AI智能体（聊天机器人服务）</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -934,30 +946,195 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>首款面向企业高管的可分离式AI决策智能体，融合实时BI数据接入、因果推断引擎与会议纪要自动生成模块</t>
+          <t>Meta于2026年5月28日宣布下月起测试的付费AI智能体订阅服务，覆盖Facebook、Instagram、WhatsApp和Meta AI，提供分级AI生成与推理能力，标志其从免费AI助手转向商业化智能体生态。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-05-29 02:04</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MuleRun</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>AI智能体框架</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>阿里云于2026年5月26日在新加坡Qwen Cloud发布会上推出的轻量级、可编排AI智能体运行时框架，专为低延迟Agent工作流设计，支持千问云Skills原生调度。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-05-28 01:56</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-05-29 02:04</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Qoder</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>智能体编程平台</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>阿里云同步发布的面向开发者的新一代智能体编程平台，支持自然语言定义Agent行为、可视化调试与一键部署至千问云，是Qwen3.7-Max的核心配套开发环境。</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-05-29 02:04</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>稀宇极智MoE大模型（未公开命名）</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>上海稀宇极智科技有限公司</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>混合专家系统（MoE）大语言模型</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>稀宇极智于2026年5月28日国务院新闻办中外记者见面会上确认发布的国内首个全自研MoE架构大模型，以不到行业巨头1%算力成本实现顶尖性能，覆盖文本理解、语音合成、视频生成及智能体全栈能力。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-05-29 02:04</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-30
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GPT-5.6</t>
+          <t>Meta One Plus / Meta One Premium</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>AI智能体（聊天机器人服务）</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -533,17 +533,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>泄露信息显示支持150万token超长上下文窗口，预计2026年6月正式发布 [重要性:高|OpenAI 的 GPT 主线模型若属实将是旗舰级重大版本更新。]</t>
+          <t>Meta于2026年5月28日宣布下月起测试的付费AI智能体订阅服务，覆盖Facebook、Instagram、WhatsApp和Meta AI，提供分级AI生成与推理能力，标志其从免费AI助手转向商业化智能体生态。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
+          <t>2026-05-29 02:04</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -553,26 +553,26 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://platform.openai.com/docs/models; 任务类型→通用对话; 开闭源→闭源; 问题: 未能确认 OpenAI 官方发布过 GPT-5.6; 现有发布时间疑似来自泄露或传闻，不应视为官方发布日期; 备注包含预测和泄露信息，建议人工核验后再录入; 模型名称包含明确版本号，形式上符合规范；但发布真实性和官方发布日期需重点复核。</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 同一条目包含两个产品/订阅档位名称，未指向单一具体模型; 类型疑似分类错误：该条目是AI智能体订阅服务/产品套餐，不是具体模型; 备注描述偏产品商业化信息，缺少模型自身技术特征; 缺少模型提供方官方页面，且无法确认其对应具体模型版本</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-29 02:03</t>
+          <t>2026-05-30 01:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Claude Mythos</t>
+          <t>dvlt</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,58 +580,66 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>大语言模型（安全增强型）</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/dvlt</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>在欧洲央行委托的红队测试中意外暴露SWIFT及三大央行结算系统漏洞，属Mythos系列新安全推理模型</t>
+          <t>HuggingFace image-to-3d</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称像系列名或代号，未指向具体模型版本; 未能确认 Anthropic 官方发布过 Claude Mythos; 备注中关于央行和 SWIFT 漏洞暴露的描述高度异常，需严格核验来源; 现有发布时间缺乏官方依据</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/dvlt)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-29 02:03</t>
+          <t>2026-05-30 01:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Claude Opus 4.8</t>
+          <t>NV-OneFormer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -641,84 +649,76 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>闭源</t>
+          <t>开源</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>多模态</t>
+          <t>未知</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/claude-opus-4-8</t>
+          <t>https://huggingface.co/nvidia/NV-OneFormer</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1000k上下文；顶级推理能力；顶级编码能力；高端定价 [重要性:高|Anthropic Claude Opus 主线高端模型若属实属于旗舰级重大版本更新。]</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://docs.anthropic.com/en/docs/about-claude/models/overview; 公司→Anthropic; 开闭源→闭源; 问题: 官网字段为第三方排行榜链接，不是 Anthropic 官方页面; 未能确认 Anthropic 官方发布过 Claude Opus 4.8; 模型发布时间需以 Anthropic 官方公告或官方模型文档为准; llm-stats.com 排行榜不应作为官方发布依据; 模型名称包含系列、档位和版本号，形式上符合规范；但该条目的发布时间、上下文长度和能力描述均需官方核验。</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NV-OneFormer)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-05-29 02:03</t>
+          <t>2026-05-30 01:58</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Qwen3.7-Max</t>
+          <t>Claude Opus 4.8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>大语言模型（代码增强型）</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -726,17 +726,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>阿里云于2026年5月20日阿里云峰会发布的面向AI Agent场景设计的新旗舰模型，在编程、推理、工具调用等能力上显著强化，支持长时间运行与多次工具调用，在Code Arena榜单中得分1541。</t>
+          <t>旗舰级编程大模型，支持200K上下文窗口，引入思维链增强机制与实时调试助手，显著提升复杂系统架构设计与错误诊断能力。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -754,19 +754,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DeepSeek-V4 Flash</t>
+          <t>GPT-5.5 Instant</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>深度求索/DeepSeek</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -781,17 +781,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>DeepSeek于2026年5月28日最新发布的高性价比推理优化版本，提供$0.14/M token定价及每日200万Token免费额度，主打高并发、低成本商用场景。</t>
+          <t>正式成为ChatGPT默认模型，医疗/法律/金融领域幻觉率较GPT-5.3降低52%，强化编码、计算机使用与深度研究能力。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -809,26 +809,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>豆包Seed 2.0 Pro</t>
+          <t>GPT-Realtime-2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>字节跳动/豆包</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>语音大模型（推理级）</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -836,17 +836,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>豆包于2026年5月28日前后正式发布升级版Seed 2.0 Pro，综合性能跻身全球前五，以$1/M token超低价格和MMMU-Pro 68.7%精度成为国产综合能力最强的商用大模型之一。</t>
+          <t>首个具备GPT-5级推理能力的实时语音模型，支持低延迟语音理解与多步语音任务规划。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -864,14 +864,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HappyHorse 1.0</t>
+          <t>GPT-Realtime-Translate</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>HappyHorse</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -883,7 +883,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>视频生成模型</t>
+          <t>语音-多模态模型（实时翻译）</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -891,17 +891,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026年5月28日官宣发布的首个专注高质量长时序视频生成的多模态基础模型，被列为2026年5月AI模型排行榜‘视频生成’唯一代表，以SOTA视频质量定位内容创作者市场。</t>
+          <t>端到端实时同传翻译模型，支持语义对齐与文化适配，延迟低于300ms，覆盖58种语言对。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -919,14 +919,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Meta One Plus / Meta One Premium</t>
+          <t>Gemini Robotics 1.5</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AI智能体（聊天机器人服务）</t>
+          <t>具身智能模型（机器人控制）</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -946,17 +946,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Meta于2026年5月28日宣布下月起测试的付费AI智能体订阅服务，覆盖Facebook、Instagram、WhatsApp和Meta AI，提供分级AI生成与推理能力，标志其从免费AI助手转向商业化智能体生态。</t>
+          <t>面向物理机器人的新一代多模态推理模型，支持跨形态技能迁移与多智能体协同决策。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -974,14 +974,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MuleRun</t>
+          <t>讯飞建筑智能体平台2.0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>科大讯飞</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -993,7 +993,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>AI智能体框架</t>
+          <t>行业智能体平台</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1001,17 +1001,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>阿里云于2026年5月26日在新加坡Qwen Cloud发布会上推出的轻量级、可编排AI智能体运行时框架，专为低延迟Agent工作流设计，支持千问云Skills原生调度。</t>
+          <t>基于全国产算力训练的建筑行业大模型+‘1+1+N’智能体架构，已落地35个可执行场景智能体，实现空调节能、会议预定、数智问答等闭环任务。</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1029,7 +1029,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Qoder</t>
+          <t>通义千问重量级新朋友（未命名）</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -1048,7 +1048,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>智能体编程平台</t>
+          <t>大语言模型（预告发布）</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1056,17 +1056,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>阿里云同步发布的面向开发者的新一代智能体编程平台，支持自然语言定义Agent行为、可视化调试与一键部署至千问云，是Qwen3.7-Max的核心配套开发环境。</t>
+          <t>阿里云峰会上正式亮相的全新旗舰模型，官方称其在全能性、深度与广度上全面对标GPT-5.5，但截至5月29日尚未公布具体型号与技术细节。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-30 01:59</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1080,61 +1080,6 @@
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>稀宇极智MoE大模型（未公开命名）</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>上海稀宇极智科技有限公司</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>混合专家系统（MoE）大语言模型</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>稀宇极智于2026年5月28日国务院新闻办中外记者见面会上确认发布的国内首个全自研MoE架构大模型，以不到行业巨头1%算力成本实现顶尖性能，覆盖文本理解、语音合成、视频生成及智能体全栈能力。</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-05-29 02:04</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-05-31
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,7 +553,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 同一条目包含两个产品/订阅档位名称，未指向单一具体模型; 类型疑似分类错误：该条目是AI智能体订阅服务/产品套餐，不是具体模型; 备注描述偏产品商业化信息，缺少模型自身技术特征; 缺少模型提供方官方页面，且无法确认其对应具体模型版本</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 同一条目包含两个产品/订阅档位名称，未指向单一具体模型; 类型疑似分类错误：该条目是AI智能体订阅服务/产品套餐，不是具体模型; 备注描述偏产品商业化信息，缺少模型自身技术特征; 缺少模型提供方官方页面，且无法确认其对应具体模型版本; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 同一条目包含两个产品/订阅档位名称，未指向单一具体模型; 类型分类错误：该条目更像AI助手订阅服务/商业化套餐，不是具体模型; 备注偏产品商业化信息，缺少模型自身技术特征; 缺少模型提供方官方页面; 无法确认其对应任何具体模型版本</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -726,7 +726,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>旗舰级编程大模型，支持200K上下文窗口，引入思维链增强机制与实时调试助手，显著提升复杂系统架构设计与错误诊断能力。</t>
+          <t>旗舰级编程大模型，支持200K上下文窗口，引入思维链增强机制与实时调试助手，显著提升复杂系统架构设计与错误诊断能力。 [重要性:高|Anthropic属于国外重点关注公司，Claude Opus若为4.x旗舰更新应属高优先级。]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→通用对话/代码生成; 官网→https://www.anthropic.com/claude; 问题: 模型名称形式符合规范：具体模型系列+版本号; 无法基于已知公开资料确认Claude Opus 4.8是否已由Anthropic官方发布; 现有备注包含较多未经核实的能力描述，建议人工复核官方公告; 保留但需重点核实发布日期、是否真实存在以及是否为官方命名。</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -781,7 +781,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>正式成为ChatGPT默认模型，医疗/法律/金融领域幻觉率较GPT-5.3降低52%，强化编码、计算机使用与深度研究能力。</t>
+          <t>正式成为ChatGPT默认模型，医疗/法律/金融领域幻觉率较GPT-5.3降低52%，强化编码、计算机使用与深度研究能力。 [重要性:高|OpenAI属于国外重点关注公司，GPT-5.5若为主线模型重大更新应为高重要性。]</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→通用对话/代码生成/智能体; 官网→https://openai.com; 问题: 模型名称形式符合规范：具体模型系列+版本/子型号; 无法基于已知公开资料确认GPT-5.5 Instant是否已由OpenAI官方发布; 备注中的医疗/法律/金融幻觉率降低52%等指标需官方来源核验; 需确认Instant是正式模型名、ChatGPT产品档位名，还是内部路由别名; 不建议因无法核实直接删除；若官方未发布，应后续人工剔除。</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -833,10 +833,14 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://openai.com/index/advancing-voice-intelligence-with-new-models-in-the-api/</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>首个具备GPT-5级推理能力的实时语音模型，支持低延迟语音理解与多步语音任务规划。</t>
+          <t>首个具备GPT-5级推理能力的实时语音模型，支持低延迟语音理解与多步语音任务规划。 [重要性:高|OpenAI实时语音模型若升级到第二代且具备推理能力，属于重点公司的重要多模态更新。]</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -856,7 +860,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→语音理解/实时语音交互; 官网→https://platform.openai.com/docs; 问题: 模型名称形式基本符合规范：具体模型名+版本号; 无法基于已知公开资料确认GPT-Realtime-2是否为OpenAI官方模型名; 备注中的GPT-5级推理能力、低延迟多步任务规划等表述需官方来源核验; 建议核查OpenAI Realtime API官方文档中是否存在该精确模型ID。</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -891,7 +895,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>端到端实时同传翻译模型，支持语义对齐与文化适配，延迟低于300ms，覆盖58种语言对。</t>
+          <t>端到端实时同传翻译模型，支持语义对齐与文化适配，延迟低于300ms，覆盖58种语言对。 [重要性:中|OpenAI重点公司的垂直实时翻译模型，若属实在语音同传场景有较高价值，但不像主线旗舰模型。]</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -911,7 +915,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→实时语音翻译/多模态翻译; 官网→https://platform.openai.com/docs; 问题: 模型名称有具体功能指向，但缺少明确版本号/型号，需确认是否为正式模型名; 无法基于已知公开资料确认GPT-Realtime-Translate是否已由OpenAI官方发布; 备注中的低于300ms延迟、58种语言对等指标需官方来源核验; 若只是Realtime API能力名称而非独立模型，应合并到对应Realtime模型条目。</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -946,7 +950,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>面向物理机器人的新一代多模态推理模型，支持跨形态技能迁移与多智能体协同决策。</t>
+          <t>面向物理机器人的新一代多模态推理模型，支持跨形态技能迁移与多智能体协同决策。 [重要性:高|Google DeepMind属于国外重点关注公司，Gemini Robotics若为机器人基础模型升级属于高价值方向。]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -966,7 +970,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Google DeepMind; 任务类型→具身智能/机器人控制; 问题: 模型名称形式符合规范：具体模型系列+版本号; 无法基于已知公开资料确认Gemini Robotics 1.5是否已由Google DeepMind官方发布; 公司名建议统一为Google DeepMind; 备注中的跨形态技能迁移、多智能体协同等能力需官方来源核验; 建议核查Google DeepMind官方博客或Gemini Robotics页面，以确认1.5版本是否真实发布。</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -1021,7 +1025,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 虽然含有2.0版本号，但名称指向的是行业智能体平台，不是具体模型; 类型不是大模型条目，属于行业应用平台/解决方案; 备注描述落地场景和架构，缺少模型自身参数、能力基准或模型版本; 缺少模型提供方官方页面</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1029,26 +1033,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>通义千问重量级新朋友（未命名）</t>
+          <t>SigenAgent v1.0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>思格新能源</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>大语言模型（预告发布）</t>
+          <t>AI智能体</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1056,17 +1060,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>阿里云峰会上正式亮相的全新旗舰模型，官方称其在全能性、深度与广度上全面对标GPT-5.5，但截至5月29日尚未公布具体型号与技术细节。</t>
+          <t>面向新能源系统的全域AI智能体，支持目标理解、自动执行与持续学习，实现从‘对话助手’到‘使命必达执行者’的跃迁。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-05-31 02:15</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1080,6 +1084,171 @@
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>悟空（Wukong）儿童陪伴人形机器人AI系统</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>中国电信</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>多模态AI智能体</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>专为3–7岁儿童设计的具身智能体，融合语音识别、视觉理解、触觉交互与情感化响应，支持自然语言问答与物理动作反馈。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-05-31 02:15</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>汽车发动机维修大数据诊断模型</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026世界智能产业博览会参展单位（未具名，属车企/工业AI联合体）</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>垂直领域大模型（工业诊断）</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>基于多源传感器与维修知识图谱构建的预测性诊断大模型，支持不拆解发动机的故障定位与维修建议生成。</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-05-31 02:15</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AgentForce 智能体中台 v2.1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>迈富时（MarketingForce）</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>AI智能体平台</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>企业级低代码智能体操作系统，支持业务人员2分钟内创建营销/销售场景专用智能体，集成NLA工作流自动生成与知识图谱驱动推理。</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-05-31 02:15</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-01
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Meta One Plus / Meta One Premium</t>
+          <t>SigenAgent v1.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>思格新能源</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>AI智能体（聊天机器人服务）</t>
+          <t>AI智能体</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -533,17 +533,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Meta于2026年5月28日宣布下月起测试的付费AI智能体订阅服务，覆盖Facebook、Instagram、WhatsApp和Meta AI，提供分级AI生成与推理能力，标志其从免费AI助手转向商业化智能体生态。</t>
+          <t>面向新能源系统的全域AI智能体，支持目标理解、自动执行与持续学习，实现从‘对话助手’到‘使命必达执行者’的跃迁。 [重要性:低|其他公司面向新能源场景的垂直智能体，行业影响力和模型级技术信息有限。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-05-31 02:15</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -553,26 +553,26 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 同一条目包含两个产品/订阅档位名称，未指向单一具体模型; 类型疑似分类错误：该条目是AI智能体订阅服务/产品套餐，不是具体模型; 备注描述偏产品商业化信息，缺少模型自身技术特征; 缺少模型提供方官方页面，且无法确认其对应具体模型版本; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 同一条目包含两个产品/订阅档位名称，未指向单一具体模型; 类型分类错误：该条目更像AI助手订阅服务/商业化套餐，不是具体模型; 备注偏产品商业化信息，缺少模型自身技术特征; 缺少模型提供方官方页面; 无法确认其对应任何具体模型版本</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://www.sigenergy.com; 任务类型→AI智能体; 公司→思格新能源（Sigenergy）; 类型→AI智能体; 问题: 发布信息待核实，未能确认是否为模型提供方官方发布; 更像行业应用智能体/产品系统，而非通用基础模型; 公司为中国企业，原始字段“国内外=国外”疑似错误; 名称包含 v1.0，形式上满足“具体产品名称+版本号”要求；但需人工核实其官方发布时间和是否应纳入模型库。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-30 01:58</t>
+          <t>2026-06-01 02:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dvlt</t>
+          <t>悟空（Wukong）儿童陪伴人形机器人AI系统</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>中国电信</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,31 +580,19 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>多模态AI智能体</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/dvlt</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace image-to-3d</t>
+          <t>专为3–7岁儿童设计的具身智能体，融合语音识别、视觉理解、触觉交互与情感化响应，支持自然语言问答与物理动作反馈。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -614,32 +602,36 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>2026-05-31 02:15</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/dvlt)</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称未包含明确版本号/型号，不满足“具体模型/产品名称+版本号/型号”规范; 更像儿童陪伴机器人产品系统，不是明确可追踪的模型版本; 公司为中国企业，原始字段“国内外=国外”疑似错误; 发布时间待核实，未能确认是否存在官方模型发布公告</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-30 01:58</t>
+          <t>2026-06-01 02:35</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NV-OneFormer</t>
+          <t>AgentForce 智能体中台 v2.1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>迈富时（MarketingForce）</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -647,78 +639,74 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>AI智能体平台</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/NV-OneFormer</t>
+          <t>https://www.marketingforce.com/</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>企业级低代码智能体操作系统，支持业务人员2分钟内创建营销/销售场景专用智能体，集成NLA工作流自动生成与知识图谱驱动推理。 [重要性:低|其他公司企业级智能体平台版本更新，偏应用平台，非基础模型或重点公司旗舰模型。]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
+          <t>2026-05-31 02:15</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NV-OneFormer)</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→AI智能体平台; 公司→迈富时（Marketingforce）; 类型→AI智能体平台; 问题: 发布信息待核实，未能确认是否为官方发布; 更像企业级智能体平台/中台产品，不是单一模型; 需注意名称可能与 Salesforce 的 Agentforce 品牌混淆，应核实提供方; 公司为中国企业，原始字段“国内外=国外”疑似错误; 名称包含 v2.1，形式上满足具体产品版本要求；但建议补充官方页面、发布公告和底层模型信息后再正式入库。</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-05-30 01:58</t>
+          <t>2026-06-01 02:35</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Claude Opus 4.8</t>
+          <t>Qwen3.7-Max</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>大语言模型（代码增强型）</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -726,17 +714,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>旗舰级编程大模型，支持200K上下文窗口，引入思维链增强机制与实时调试助手，显著提升复杂系统架构设计与错误诊断能力。 [重要性:高|Anthropic属于国外重点关注公司，Claude Opus若为4.x旗舰更新应属高优先级。]</t>
+          <t>通义千问在2026年5月20日阿里云峰会正式发布的旗舰级大模型，编程能力全球第二（Code Arena 1541分），支持超1000次工具调用的长程智能体任务，推理速度较前代提升10倍。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -746,7 +734,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→通用对话/代码生成; 官网→https://www.anthropic.com/claude; 问题: 模型名称形式符合规范：具体模型系列+版本号; 无法基于已知公开资料确认Claude Opus 4.8是否已由Anthropic官方发布; 现有备注包含较多未经核实的能力描述，建议人工复核官方公告; 保留但需重点核实发布日期、是否真实存在以及是否为官方命名。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -754,26 +742,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GPT-5.5 Instant</t>
+          <t>Doubao-Seed-2.0-Pro</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>字节跳动/豆包</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>原生多模态智能体</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -781,17 +769,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>正式成为ChatGPT默认模型，医疗/法律/金融领域幻觉率较GPT-5.3降低52%，强化编码、计算机使用与深度研究能力。 [重要性:高|OpenAI属于国外重点关注公司，GPT-5.5若为主线模型重大更新应为高重要性。]</t>
+          <t>豆包2.0系列旗舰版本，实现视频、图像、音频、文本的原生统一理解与视听联合推理，完成从对话AI到‘实体智能体’的范式跃迁。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -801,7 +789,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→通用对话/代码生成/智能体; 官网→https://openai.com; 问题: 模型名称形式符合规范：具体模型系列+版本/子型号; 无法基于已知公开资料确认GPT-5.5 Instant是否已由OpenAI官方发布; 备注中的医疗/法律/金融幻觉率降低52%等指标需官方来源核验; 需确认Instant是正式模型名、ChatGPT产品档位名，还是内部路由别名; 不建议因无法核实直接删除；若官方未发布，应后续人工剔除。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -809,7 +797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GPT-Realtime-2</t>
+          <t>GPT-5.5 Instant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -828,29 +816,25 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>语音大模型（推理级）</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://openai.com/index/advancing-voice-intelligence-with-new-models-in-the-api/</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>首个具备GPT-5级推理能力的实时语音模型，支持低延迟语音理解与多步语音任务规划。 [重要性:高|OpenAI实时语音模型若升级到第二代且具备推理能力，属于重点公司的重要多模态更新。]</t>
+          <t>GPT-5.5系列默认部署版本，取代GPT-5.3成为ChatGPT主力模型，医疗/法律/金融领域幻觉率下降52%，显著增强编码与计算机使用能力。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -860,7 +844,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→语音理解/实时语音交互; 官网→https://platform.openai.com/docs; 问题: 模型名称形式基本符合规范：具体模型名+版本号; 无法基于已知公开资料确认GPT-Realtime-2是否为OpenAI官方模型名; 备注中的GPT-5级推理能力、低延迟多步任务规划等表述需官方来源核验; 建议核查OpenAI Realtime API官方文档中是否存在该精确模型ID。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -868,7 +852,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GPT-Realtime-Translate</t>
+          <t>GPT-Realtime-2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -887,7 +871,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>语音-多模态模型（实时翻译）</t>
+          <t>语音推理模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -895,7 +879,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>端到端实时同传翻译模型，支持语义对齐与文化适配，延迟低于300ms，覆盖58种语言对。 [重要性:中|OpenAI重点公司的垂直实时翻译模型，若属实在语音同传场景有较高价值，但不像主线旗舰模型。]</t>
+          <t>首个具备GPT-5级推理能力的实时语音模型，支持语音输入下的多步逻辑推演与上下文保持。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -905,7 +889,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -915,7 +899,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→实时语音翻译/多模态翻译; 官网→https://platform.openai.com/docs; 问题: 模型名称有具体功能指向，但缺少明确版本号/型号，需确认是否为正式模型名; 无法基于已知公开资料确认GPT-Realtime-Translate是否已由OpenAI官方发布; 备注中的低于300ms延迟、58种语言对等指标需官方来源核验; 若只是Realtime API能力名称而非独立模型，应合并到对应Realtime模型条目。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -923,14 +907,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gemini Robotics 1.5</t>
+          <t>GPT-Realtime-Translate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -942,7 +926,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>具身智能模型（机器人控制）</t>
+          <t>语音翻译模型</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -950,17 +934,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>面向物理机器人的新一代多模态推理模型，支持跨形态技能迁移与多智能体协同决策。 [重要性:高|Google DeepMind属于国外重点关注公司，Gemini Robotics若为机器人基础模型升级属于高价值方向。]</t>
+          <t>端到端实时同传翻译模型，支持低延迟、高保真跨语言语义对齐，已集成至Teams和Zoom企业插件。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -970,7 +954,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Google DeepMind; 任务类型→具身智能/机器人控制; 问题: 模型名称形式符合规范：具体模型系列+版本号; 无法基于已知公开资料确认Gemini Robotics 1.5是否已由Google DeepMind官方发布; 公司名建议统一为Google DeepMind; 备注中的跨形态技能迁移、多智能体协同等能力需官方来源核验; 建议核查Google DeepMind官方博客或Gemini Robotics页面，以确认1.5版本是否真实发布。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -978,26 +962,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>讯飞建筑智能体平台2.0</t>
+          <t>Gemini Robotics 1.5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>科大讯飞</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>行业智能体平台</t>
+          <t>具身智能模型</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1005,17 +989,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>基于全国产算力训练的建筑行业大模型+‘1+1+N’智能体架构，已落地35个可执行场景智能体，实现空调节能、会议预定、数智问答等闭环任务。</t>
+          <t>专为机器人设计的下一代世界模型，支持跨形态技能迁移与多智能体协作规划，已在波士顿动力Atlas及UBTECH Walker X平台实测部署。</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-30 01:59</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1025,7 +1009,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 虽然含有2.0版本号，但名称指向的是行业智能体平台，不是具体模型; 类型不是大模型条目，属于行业应用平台/解决方案; 备注描述落地场景和架构，缺少模型自身参数、能力基准或模型版本; 缺少模型提供方官方页面</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1033,26 +1017,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SigenAgent v1.0</t>
+          <t>DeepSeek R1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>思格新能源</t>
+          <t>深度求索/DeepSeek</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>AI智能体</t>
+          <t>强化对齐大模型</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1060,17 +1044,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>面向新能源系统的全域AI智能体，支持目标理解、自动执行与持续学习，实现从‘对话助手’到‘使命必达执行者’的跃迁。</t>
+          <t>基于RLHF+Test-time Scaling双路径优化的推理增强模型，在MMLU-Pro与AgentBench上刷新国产模型纪录，强调‘可解释决策链’输出。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-31 02:15</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1088,26 +1072,26 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>悟空（Wukong）儿童陪伴人形机器人AI系统</t>
+          <t>Kimi-Max-2605</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>中国电信</t>
+          <t>月之暗面/Kimi</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>多模态AI智能体</t>
+          <t>长上下文智能体</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1115,17 +1099,17 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>专为3–7岁儿童设计的具身智能体，融合语音识别、视觉理解、触觉交互与情感化响应，支持自然语言问答与物理动作反馈。</t>
+          <t>支持200万token上下文的轻量化智能体框架，专为法律文书分析、科研文献综述等专业场景优化，已接入国家知识产权局政务AI中台。</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-31 02:15</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1143,26 +1127,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>汽车发动机维修大数据诊断模型</t>
+          <t>GLM-5-AllSpark</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026世界智能产业博览会参展单位（未具名，属车企/工业AI联合体）</t>
+          <t>智谱AI/GLM</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>垂直领域大模型（工业诊断）</t>
+          <t>全模态生成模型</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1170,17 +1154,17 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>基于多源传感器与维修知识图谱构建的预测性诊断大模型，支持不拆解发动机的故障定位与维修建议生成。</t>
+          <t>GLM系列首款支持‘文本→3D网格+物理仿真参数+音效轨迹’联合生成的Diffusion 3.0原生模型，面向工业数字孪生场景发布。</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-31 02:15</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1198,26 +1182,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AgentForce 智能体中台 v2.1</t>
+          <t>SenseNova 6.0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>迈富时（MarketingForce）</t>
+          <t>商汤科技</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>AI智能体平台</t>
+          <t>多模态基础模型</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1225,17 +1209,17 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>企业级低代码智能体操作系统，支持业务人员2分钟内创建营销/销售场景专用智能体，集成NLA工作流自动生成与知识图谱驱动推理。</t>
+          <t>覆盖视觉、语音、文本、雷达点云的八模态统一架构模型，首次将毫米波雷达信号纳入大模型感知通路，用于L4级车路协同系统。</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-31 02:15</t>
+          <t>2026-06-01 02:36</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-03
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GPT-5.6</t>
+          <t>CircularNet</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,58 +521,66 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>大语言模型</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/google/CircularNet</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>泄露信息显示支持150万token超长上下文窗口，预计2026年6月正式发布 [重要性:高|OpenAI 的 GPT 主线模型若属实将是旗舰级重大版本更新。]</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://platform.openai.com/docs/models; 任务类型→通用对话; 开闭源→闭源; 问题: 未能确认 OpenAI 官方发布过 GPT-5.6; 现有发布时间疑似来自泄露或传闻，不应视为官方发布日期; 备注包含预测和泄露信息，建议人工核验后再录入; 模型名称包含明确版本号，形式上符合规范；但发布真实性和官方发布日期需重点复核。</t>
+          <t>HuggingFace 已核实(google/CircularNet) · apache-2.0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-29 02:03</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Claude Mythos</t>
+          <t>4D-RGPT-8B</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,145 +588,137 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8B</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>大语言模型（安全增强型）</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/4D-RGPT-8B</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>在欧洲央行委托的红队测试中意外暴露SWIFT及三大央行结算系统漏洞，属Mythos系列新安全推理模型</t>
+          <t>HuggingFace video-text-to-text</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-28 01:56</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称像系列名或代号，未指向具体模型版本; 未能确认 Anthropic 官方发布过 Claude Mythos; 备注中关于央行和 SWIFT 漏洞暴露的描述高度异常，需严格核验来源; 现有发布时间缺乏官方依据</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/4D-RGPT-8B)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-29 02:03</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Claude Opus 4.8</t>
+          <t>Qwen3.7-Plus</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>多模态</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/claude-opus-4-8</t>
-        </is>
-      </c>
+          <t>多模态智能体模型</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1000k上下文；顶级推理能力；顶级编码能力；高端定价 [重要性:高|Anthropic Claude Opus 主线高端模型若属实属于旗舰级重大版本更新。]</t>
+          <t>阿里发布的全新多模态智能体模型，面向复杂任务编排与具身交互优化。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>是</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://docs.anthropic.com/en/docs/about-claude/models/overview; 公司→Anthropic; 开闭源→闭源; 问题: 官网字段为第三方排行榜链接，不是 Anthropic 官方页面; 未能确认 Anthropic 官方发布过 Claude Opus 4.8; 模型发布时间需以 Anthropic 官方公告或官方模型文档为准; llm-stats.com 排行榜不应作为官方发布依据; 模型名称包含系列、档位和版本号，形式上符合规范；但该条目的发布时间、上下文长度和能力描述均需官方核验。</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-05-29 02:03</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Qwen3.7-Max</t>
+          <t>MAI-Thinking-1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>旗舰推理大语言模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -726,17 +726,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>阿里云于2026年5月20日阿里云峰会发布的面向AI Agent场景设计的新旗舰模型，在编程、推理、工具调用等能力上显著强化，支持长时间运行与多次工具调用，在Code Arena榜单中得分1541。</t>
+          <t>微软MAI家族首款中型自研推理模型，零蒸馏训练，在软件工程测试中性能媲美Sonnet 4.6。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -754,26 +754,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DeepSeek-V4 Flash</t>
+          <t>MAI-Code-1-Flash</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>深度求索/DeepSeek</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>编程专用agentic模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -781,17 +781,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>DeepSeek于2026年5月28日最新发布的高性价比推理优化版本，提供$0.14/M token定价及每日200万Token免费额度，主打高并发、低成本商用场景。</t>
+          <t>50亿参数高效编码模型，深度集成GitHub Copilot与VS Code，专为微软技术栈优化。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -809,26 +809,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>豆包Seed 2.0 Pro</t>
+          <t>DobotWAM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>字节跳动/豆包</t>
+          <t>越疆科技</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>具身智能体大模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -836,17 +836,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>豆包于2026年5月28日前后正式发布升级版Seed 2.0 Pro，综合性能跻身全球前五，以$1/M token超低价格和MMMU-Pro 68.7%精度成为国产综合能力最强的商用大模型之一。</t>
+          <t>面向机器人操作的具身大模型，在LIBERO基准登顶第一，任务成功率99.25%。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -864,26 +864,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HappyHorse 1.0</t>
+          <t>MiniMax M3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>HappyHorse</t>
+          <t>MiniMax/海螺</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>视频生成模型</t>
+          <t>多模态大模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -891,17 +891,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026年5月28日官宣发布的首个专注高质量长时序视频生成的多模态基础模型，被列为2026年5月AI模型排行榜‘视频生成’唯一代表，以SOTA视频质量定位内容创作者市场。</t>
+          <t>京东云率先上线的MiniMax最新多模态基础模型，支持图文音视频联合理解与生成。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -919,14 +919,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Meta One Plus / Meta One Premium</t>
+          <t>LobsterAI Image-Video Matrix</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>LobsterAI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -938,7 +938,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AI智能体（聊天机器人服务）</t>
+          <t>图像/视频生成大模型矩阵</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -946,17 +946,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Meta于2026年5月28日宣布下月起测试的付费AI智能体订阅服务，覆盖Facebook、Instagram、WhatsApp和Meta AI，提供分级AI生成与推理能力，标志其从免费AI助手转向商业化智能体生态。</t>
+          <t>LobsterAI发布的多分辨率、多时长视频与高保真图像协同生成模型集合。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-29 02:04</t>
+          <t>2026-06-03 02:40</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -970,171 +970,6 @@
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MuleRun</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>阿里巴巴/通义</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>AI智能体框架</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>阿里云于2026年5月26日在新加坡Qwen Cloud发布会上推出的轻量级、可编排AI智能体运行时框架，专为低延迟Agent工作流设计，支持千问云Skills原生调度。</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-05-29 02:04</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Qoder</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>阿里巴巴/通义</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>智能体编程平台</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>阿里云同步发布的面向开发者的新一代智能体编程平台，支持自然语言定义Agent行为、可视化调试与一键部署至千问云，是Qwen3.7-Max的核心配套开发环境。</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2026-05-29 02:04</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>稀宇极智MoE大模型（未公开命名）</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>上海稀宇极智科技有限公司</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>混合专家系统（MoE）大语言模型</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>稀宇极智于2026年5月28日国务院新闻办中外记者见面会上确认发布的国内首个全自研MoE架构大模型，以不到行业巨头1%算力成本实现顶尖性能，覆盖文本理解、语音合成、视频生成及智能体全栈能力。</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-05-29 02:04</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-04
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CircularNet</t>
+          <t>LobsterAI Image-Video Matrix</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>LobsterAI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,31 +521,19 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>图像/视频生成大模型矩阵</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/google/CircularNet</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>LobsterAI发布的多分辨率、多时长视频与高保真图像协同生成模型集合。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -555,32 +543,36 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+          <t>2026-06-03 02:40</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>HuggingFace 已核实(google/CircularNet) · apache-2.0</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称指向模型矩阵/模型集合，不是具体的模型/产品名称 + 版本号/型号; 未能基于已知公开信息确认其为官方发布的具体模型</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4D-RGPT-8B</t>
+          <t>MAI-Code-1-Flash</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -588,82 +580,66 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>8B</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>代码生成大语言模型</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/4D-RGPT-8B</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace video-text-to-text</t>
+          <t>微软在 Build 2026 大会上发布的首款自研代码生成模型，支持自然语言到应用程序/网站源代码的端到端生成，已集成至 GitHub Copilot 和 VS Code。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>2026-06-04 02:36</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/4D-RGPT-8B)</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-06-03 02:40</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Qwen3.7-Plus</t>
+          <t>MAI-Thinking-1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>多模态智能体模型</t>
+          <t>推理型大语言模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -671,17 +647,17 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>阿里发布的全新多模态智能体模型，面向复杂任务编排与具身交互优化。</t>
+          <t>微软发布的旗舰推理模型，在编码基准测试中性能媲美 Anthropic Claude Sonnet 4.6，为微软新一代智能体核心推理引擎。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -699,7 +675,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MAI-Thinking-1</t>
+          <t>MAI-Vision-1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -718,7 +694,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>旗舰推理大语言模型</t>
+          <t>多模态视觉理解模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -726,17 +702,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>微软MAI家族首款中型自研推理模型，零蒸馏训练，在软件工程测试中性能媲美Sonnet 4.6。</t>
+          <t>微软在 Build 2026 发布的视觉基础模型，支持图像、文档、图表等复杂视觉输入的语义解析与跨模态推理，专为智能体环境感知优化。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -754,7 +730,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAI-Code-1-Flash</t>
+          <t>MAI-Speech-1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -773,7 +749,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>编程专用agentic模型</t>
+          <t>语音大语言模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -781,17 +757,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>50亿参数高效编码模型，深度集成GitHub Copilot与VS Code，专为微软技术栈优化。</t>
+          <t>微软新发布的低延迟、高保真语音交互模型，支持实时流式语音理解与生成，深度集成于 Windows Copilot+ 设备及 Teams 智能会议场景。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -809,14 +785,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DobotWAM</t>
+          <t>MAI-Multimodal-Agent-1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>越疆科技</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -828,7 +804,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>具身智能体大模型</t>
+          <t>自主智能体（Agent）系统</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -836,17 +812,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>面向机器人操作的具身大模型，在LIBERO基准登顶第一，任务成功率99.25%。</t>
+          <t>基于 MAI 系列模型构建的首个端到端可执行智能体框架，支持任务规划、工具调用、Web IQ 搜索协同与长期记忆，面向企业自动化场景开放 SDK。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -864,26 +840,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MiniMax M3</t>
+          <t>Web IQ</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MiniMax/海螺</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>多模态大模型</t>
+          <t>AI智能体专用搜索 API 服务</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -891,17 +867,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>京东云率先上线的MiniMax最新多模态基础模型，支持图文音视频联合理解与生成。</t>
+          <t>微软推出的面向 AI 智能体的语义化网络检索服务，提供带 grounding 的结构化网页、新闻、图片、视频内容，非面向人类的传统搜索引擎。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -919,14 +895,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LobsterAI Image-Video Matrix</t>
+          <t>Mayo-Medical-LLM (codename: MedSage)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LobsterAI</t>
+          <t>Mayo Clinic &amp; Microsoft</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -938,7 +914,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>图像/视频生成大模型矩阵</t>
+          <t>医疗垂直领域大语言模型</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -946,17 +922,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>LobsterAI发布的多分辨率、多时长视频与高保真图像协同生成模型集合。</t>
+          <t>梅奥诊所与微软联合发布、由梅奥持有主权的临床级 AI 模型，基于去标识化真实世界健康数据训练，专注临床推理与诊疗辅助，尚未开源或商用。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-05
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LobsterAI Image-Video Matrix</t>
+          <t>MAI-Multimodal-Agent-1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LobsterAI</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>图像/视频生成大模型矩阵</t>
+          <t>自主智能体（Agent）系统</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -533,17 +533,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>LobsterAI发布的多分辨率、多时长视频与高保真图像协同生成模型集合。</t>
+          <t>基于 MAI 系列模型构建的首个端到端可执行智能体框架，支持任务规划、工具调用、Web IQ 搜索协同与长期记忆，面向企业自动化场景开放 SDK。 [重要性:中|若属实，这是微软面向企业自动化的多模态智能体框架，具备一定平台级价值，但公开信息仍需人工核实。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-03 02:40</t>
+          <t>2026-06-04 02:36</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -553,26 +553,26 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称指向模型矩阵/模型集合，不是具体的模型/产品名称 + 版本号/型号; 未能基于已知公开信息确认其为官方发布的具体模型</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→自主智能体/多模态智能体; 公司→Microsoft AI; 类型→自主智能体（Agent）系统; 问题: 名称包含明确型号/版本号，形式上符合具体模型或系统名称规范; 当前信息显示更像智能体系统/框架，而非传统基础模型，需确认是否应纳入模型库; 发布时间为2026-06-03，处于本次追踪窗口附近，可宽松保留; 核实情况为待核实，建议人工查验微软官方发布源; 未能基于已知可靠公开知识确认该名称及发布日期，建议以 Microsoft AI 官方博客、Azure AI 文档或 GitHub/SDK 发布记录为准。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-04 02:35</t>
+          <t>2026-06-05 02:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MAI-Code-1-Flash</t>
+          <t>ArtiFixer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,42 +580,54 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>代码生成大语言模型</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/ArtiFixer</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>微软在 Build 2026 大会上发布的首款自研代码生成模型，支持自然语言到应用程序/网站源代码的端到端生成，已集成至 GitHub Copilot 和 VS Code。</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr"/>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/ArtiFixer)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-06-05 02:10</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -639,7 +651,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>推理型大语言模型</t>
+          <t>大语言模型（推理专用）</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -647,7 +659,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>微软发布的旗舰推理模型，在编码基准测试中性能媲美 Anthropic Claude Sonnet 4.6，为微软新一代智能体核心推理引擎。</t>
+          <t>微软在Build 2026大会上发布的旗舰推理模型，在编码基准测试中与Anthropic Claude Sonnet 4.6持平。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -657,7 +669,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
+          <t>2026-06-05 02:11</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -675,7 +687,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MAI-Vision-1</t>
+          <t>MAI-Code-1-Flash</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -694,7 +706,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>多模态视觉理解模型</t>
+          <t>代码大语言模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -702,7 +714,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>微软在 Build 2026 发布的视觉基础模型，支持图像、文档、图表等复杂视觉输入的语义解析与跨模态推理，专为智能体环境感知优化。</t>
+          <t>微软首款AI编程模型，50亿参数，面向VS Code/GitHub Copilot个人版，高性价比，Token消耗较Claude Haiku 4.5最高降低60%。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -712,7 +724,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
+          <t>2026-06-05 02:11</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -730,7 +742,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAI-Speech-1</t>
+          <t>MAI-Vision-1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -749,7 +761,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>语音大语言模型</t>
+          <t>多模态模型（视觉理解）</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -757,7 +769,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>微软新发布的低延迟、高保真语音交互模型，支持实时流式语音理解与生成，深度集成于 Windows Copilot+ 设备及 Teams 智能会议场景。</t>
+          <t>微软Build 2026发布的全栈模型之一，支持细粒度图像-文本对齐与跨模态推理，已集成至Windows Copilot+生态。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -767,7 +779,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
+          <t>2026-06-05 02:11</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -785,7 +797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MAI-Multimodal-Agent-1</t>
+          <t>MAI-Speech-1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -804,7 +816,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>自主智能体（Agent）系统</t>
+          <t>语音大模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -812,7 +824,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>基于 MAI 系列模型构建的首个端到端可执行智能体框架，支持任务规划、工具调用、Web IQ 搜索协同与长期记忆，面向企业自动化场景开放 SDK。</t>
+          <t>低延迟、高保真端到端语音合成与识别模型，支持实时双语会议转录与智能摘要，首发搭载于Surface RTX Spark Dev Box。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -822,7 +834,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
+          <t>2026-06-05 02:11</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -840,7 +852,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Web IQ</t>
+          <t>MAI-Multimodal-1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -859,7 +871,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>AI智能体专用搜索 API 服务</t>
+          <t>多模态大模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -867,7 +879,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>微软推出的面向 AI 智能体的语义化网络检索服务，提供带 grounding 的结构化网页、新闻、图片、视频内容，非面向人类的传统搜索引擎。</t>
+          <t>微软七款新模型之一，统一架构支持文本、图像、音频、代码联合输入输出，面向企业级Copilot Agent工作流。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -877,7 +889,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
+          <t>2026-06-05 02:11</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -895,14 +907,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mayo-Medical-LLM (codename: MedSage)</t>
+          <t>MAI-Agent-Core-v1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mayo Clinic &amp; Microsoft</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -914,7 +926,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>医疗垂直领域大语言模型</t>
+          <t>智能体框架/运行时</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -922,7 +934,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>梅奥诊所与微软联合发布、由梅奥持有主权的临床级 AI 模型，基于去标识化真实世界健康数据训练，专注临床推理与诊疗辅助，尚未开源或商用。</t>
+          <t>微软发布的轻量级Agentic AI运行时，原生支持PRAR循环（感知-推理-行动-反思），深度集成Windows Terminal与WSL2。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -932,7 +944,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
+          <t>2026-06-05 02:11</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -946,6 +958,61 @@
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MAI-Toolformer-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>工具调用增强模型</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>专为自动工具发现、API Schema理解与安全工具链编排优化的微调模型，作为MAI-Agent-Core-v1的默认控制器。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-05 02:11</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-06
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MAI-Multimodal-Agent-1</t>
+          <t>gemma-4-12B-it-qat-w4a16-ct</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,58 +521,70 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>12B</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>自主智能体（Agent）系统</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/google/gemma-4-12B-it-qat-w4a16-ct</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>基于 MAI 系列模型构建的首个端到端可执行智能体框架，支持任务规划、工具调用、Web IQ 搜索协同与长期记忆，面向企业自动化场景开放 SDK。 [重要性:中|若属实，这是微软面向企业自动化的多模态智能体框架，具备一定平台级价值，但公开信息仍需人工核实。]</t>
+          <t>HuggingFace any-to-any</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-04 02:36</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 任务类型→自主智能体/多模态智能体; 公司→Microsoft AI; 类型→自主智能体（Agent）系统; 问题: 名称包含明确型号/版本号，形式上符合具体模型或系统名称规范; 当前信息显示更像智能体系统/框架，而非传统基础模型，需确认是否应纳入模型库; 发布时间为2026-06-03，处于本次追踪窗口附近，可宽松保留; 核实情况为待核实，建议人工查验微软官方发布源; 未能基于已知可靠公开知识确认该名称及发布日期，建议以 Microsoft AI 官方博客、Azure AI 文档或 GitHub/SDK 发布记录为准。</t>
+          <t>HuggingFace 已核实(google/gemma-4-12B-it-qat-w4a16-ct) · 参数量=13B · apache-2.0 · any-to-any</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-05 02:10</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ArtiFixer</t>
+          <t>Cosmos 3 (Super/Base/Tiny)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -580,66 +592,54 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>全模态物理AI基础模型</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/ArtiFixer</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>全球首款完全开源的文本/图像/视频/音频/动作五模态物理AI模型，原生支持重力、摩擦、碰撞等物理规则建模，基于混合Transformer（MoT）架构。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>2026-06-06 02:02</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/ArtiFixer)</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-06-05 02:10</t>
-        </is>
-      </c>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MAI-Thinking-1</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -651,7 +651,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>大语言模型（推理专用）</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -659,17 +659,17 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>微软在Build 2026大会上发布的旗舰推理模型，在编码基准测试中与Anthropic Claude Sonnet 4.6持平。</t>
+          <t>千亿参数Dense架构LLM，MMLU-Pro达89.5分，支持INT4量化在RTX 5090上实时推理（首Token延迟低至180ms），面向消费级GPU优化。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-05 02:11</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -687,26 +687,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MAI-Code-1-Flash</t>
+          <t>MiniMax M3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>代码大语言模型</t>
+          <t>多模态大语言模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -714,17 +714,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>微软首款AI编程模型，50亿参数，面向VS Code/GitHub Copilot个人版，高性价比，Token消耗较Claude Haiku 4.5最高降低60%。</t>
+          <t>国内首个同时具备前沿Coding能力、1M超长上下文、原生多模态的国产大模型，采用自研MSA稀疏注意力架构，SWE-Bench Pro超越GPT-5.5。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-05 02:11</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -742,14 +742,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAI-Vision-1</t>
+          <t>Qwen3.7-Plus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Alibaba (Tongyi Lab)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -761,7 +761,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>多模态模型（视觉理解）</t>
+          <t>多模态智能体模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -769,17 +769,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>微软Build 2026发布的全栈模型之一，支持细粒度图像-文本对齐与跨模态推理，已集成至Windows Copilot+生态。</t>
+          <t>主打‘看想做做验’一体化智能体能力，可连续11小时自主开发App，覆盖需求理解、代码生成、测试验证等全流程项目级任务。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-05 02:11</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MAI-Speech-1</t>
+          <t>MAI-Code-1-Flash</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -816,7 +816,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>语音大模型</t>
+          <t>代码推理模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -824,17 +824,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>低延迟、高保真端到端语音合成与识别模型，支持实时双语会议转录与智能摘要，首发搭载于Surface RTX Spark Dev Box。</t>
+          <t>微软Build 2026发布的开源高级代码推理模型，专为复杂工程级代码生成与调试优化，支持多文件上下文协同推理。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-05 02:11</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -852,7 +852,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAI-Multimodal-1</t>
+          <t>MAI Thinking 1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -871,7 +871,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>多模态大模型</t>
+          <t>深度推理模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -879,17 +879,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>微软七款新模型之一，统一架构支持文本、图像、音频、代码联合输入输出，面向企业级Copilot Agent工作流。</t>
+          <t>微软自研的深度链式推理（Chain-of-Thought）增强模型，面向数学证明、逻辑规划与跨文档复杂决策任务。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-05 02:11</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -907,26 +907,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MAI-Agent-Core-v1</t>
+          <t>Kimi K2.6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Moonshot AI (月之暗面)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>智能体框架/运行时</t>
+          <t>开源多模态智能体模型</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -934,17 +934,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>微软发布的轻量级Agentic AI运行时，原生支持PRAR循环（感知-推理-行动-反思），深度集成Windows Terminal与WSL2。</t>
+          <t>Kimi K2系列最新版本，强化编程与Agent集群能力，支持动态生成多个子Agent并行协作，已开源（发布时间在搜索窗口前，但为截至2026-06-05最新稳定版，广泛报道于6月初技术综述中）。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-06-05 02:11</t>
+          <t>2026-06-06 02:02</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -958,61 +958,6 @@
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MAI-Toolformer-1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>工具调用增强模型</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>专为自动工具发现、API Schema理解与安全工具链编排优化的微调模型，作为MAI-Agent-Core-v1的默认控制器。</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-06-05 02:11</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-07
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,10 +601,14 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://build.nvidia.com</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>全球首款完全开源的文本/图像/视频/音频/动作五模态物理AI模型，原生支持重力、摩擦、碰撞等物理规则建模，基于混合Transformer（MoT）架构。</t>
+          <t>全球首款完全开源的文本/图像/视频/音频/动作五模态物理AI模型，原生支持重力、摩擦、碰撞等物理规则建模，基于混合Transformer（MoT）架构。 [重要性:高|NVIDIA物理AI/世界模型若为重大版本更新，具备较高行业关注度和技术价值。]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -624,7 +628,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://www.nvidia.com/en-us/ai/cosmos/; 任务类型→物理AI/世界模型; 备注→物理AI世界基础模型；多模态生成与理解；面向机器人与仿真场景；开源情况需核实; 问题: 模型名称包含多个变体Super/Base/Tiny，建议拆分为独立模型条目或明确主模型与子型号; 未能基于已知公开资料核实Cosmos 3于2026-06-01官方发布; 备注中“全球首款完全开源”“五模态”等表述需官方来源核实; 开源标注需复核，NVIDIA Cosmos系列可能存在开放权重、开放许可与完全开源的区别; 名称具备版本号，不属于产品泛称；如确为2026年6月发布，应保留。</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -656,10 +660,14 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://build.nvidia.com</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>千亿参数Dense架构LLM，MMLU-Pro达89.5分，支持INT4量化在RTX 5090上实时推理（首Token延迟低至180ms），面向消费级GPU优化。</t>
+          <t>千亿参数Dense架构LLM，MMLU-Pro达89.5分，支持INT4量化在RTX 5090上实时推理（首Token延迟低至180ms），面向消费级GPU优化。 [重要性:中|NVIDIA属于国外优秀关注公司，Nemotron若为新一代大模型更新值得关注。]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -679,7 +687,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://www.nvidia.com/en-us/ai-data-science/foundation-models/nemotron/; 任务类型→通用对话/推理; 备注→Nemotron系列大语言模型；面向推理与企业AI应用；参数规模、Benchmark与消费级GPU优化能力需官方核实; 问题: 未能基于已知公开资料核实Nemotron 3 Ultra于2026-06-01官方发布; “千亿参数Dense架构”“MMLU-Pro 89.5”“RTX 5090实时推理”等具体指标需官方来源核实; 名称具备版本/型号，不属于产品泛称; 建议人工核查NVIDIA官方博客、NVIDIA NIM/Build平台及技术报告。</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -714,7 +722,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>国内首个同时具备前沿Coding能力、1M超长上下文、原生多模态的国产大模型，采用自研MSA稀疏注意力架构，SWE-Bench Pro超越GPT-5.5。</t>
+          <t>国内首个同时具备前沿Coding能力、1M超长上下文、原生多模态的国产大模型，采用自研MSA稀疏注意力架构，SWE-Bench Pro超越GPT-5.5。 [重要性:高|MiniMax属于国内重点关注公司，若M3为旗舰级多模态大模型则属于重大版本更新。]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -734,7 +742,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→MiniMax; 官网→https://www.minimax.io/; 任务类型→通用对话/多模态/代码生成; 备注→MiniMax系列多模态大模型；长上下文、代码能力与Agent能力需官方核实; 问题: 未能基于已知公开资料核实MiniMax M3于2026-06-01官方发布; “国内首个”“SWE-Bench Pro超越GPT-5.5”等强断言需官方或权威评测来源核实; 名称具备版本号，不属于产品泛称; 如官方确认发布时间为2026年，应保留；当前描述存在明显营销化和未核实Benchmark风险。</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -766,10 +774,14 @@
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://tongyi.aliyun.com/</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>主打‘看想做做验’一体化智能体能力，可连续11小时自主开发App，覆盖需求理解、代码生成、测试验证等全流程项目级任务。</t>
+          <t>主打‘看想做做验’一体化智能体能力，可连续11小时自主开发App，覆盖需求理解、代码生成、测试验证等全流程项目级任务。 [重要性:高|Qwen属于国内重点关注公司的核心模型系列，若为3.7代Plus更新则具备高关注价值。]</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -789,7 +801,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→阿里巴巴/通义千问; 官网→https://qwenlm.github.io/; 任务类型→通用对话/多模态/智能体; 备注→Qwen系列Plus版本；面向通用对话、代码与智能体任务；具体长程Agent能力需官方核实; 问题: 公司名建议统一为“阿里巴巴/通义千问”; 原始数据中“国内外”标为国外，与阿里巴巴/通义千问不符，应为国内; 未能基于已知公开资料核实Qwen3.7-Plus于2026-06-02官方发布; 类型标为“多模态智能体模型”需复核，Plus版本可能是通用大模型而非专门智能体模型; 备注中“连续11小时自主开发App”等能力描述需官方评测或演示来源核实; 名称具备版本/型号，不属于产品泛称；建议核查Qwen官方博客、GitHub和模型卡。</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -824,7 +836,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>微软Build 2026发布的开源高级代码推理模型，专为复杂工程级代码生成与调试优化，支持多文件上下文协同推理。</t>
+          <t>微软Build 2026发布的开源高级代码推理模型，专为复杂工程级代码生成与调试优化，支持多文件上下文协同推理。 [重要性:中|微软自研代码模型若属实，在代码生成领域具有较高应用价值，但不在重点关注公司清单内。]</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -844,7 +856,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Microsoft AI; 任务类型→代码生成/代码推理; 备注→代码推理模型；面向复杂工程级代码生成、调试与多文件上下文处理；开源情况需官方核实; 问题: 未能基于已知公开资料核实MAI-Code-1-Flash于2026-06-02官方发布; “Build 2026发布”“开源高级代码推理模型”等信息需微软官方公告核实; 开闭源标注缺失且备注称开源，建议补充并核实许可证; 名称具备版本/型号，不属于产品泛称; 建议核查Microsoft AI Blog、Build大会公告、Azure AI Foundry模型目录和GitHub。</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -879,7 +891,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>微软自研的深度链式推理（Chain-of-Thought）增强模型，面向数学证明、逻辑规划与跨文档复杂决策任务。</t>
+          <t>微软自研的深度链式推理（Chain-of-Thought）增强模型，面向数学证明、逻辑规划与跨文档复杂决策任务。 [重要性:中|微软自研推理模型若属实属于重要厂商在推理方向的更新，具备中等以上关注价值。]</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -899,7 +911,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Microsoft AI; 任务类型→深度推理/通用对话; 备注→深度推理模型；面向数学、逻辑规划与复杂决策；具体推理机制和性能需官方核实; 问题: 未能基于已知公开资料核实MAI Thinking 1于2026-06-02官方发布; 模型命名是否应为“MAI-Thinking-1”或其他官方格式需复核; 备注中“深度链式推理增强”等技术描述需官方技术报告核实; 名称具备版本号，不属于产品泛称; 建议核查Microsoft AI官方博客、Azure AI Foundry及Build 2026发布资料。</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -934,7 +946,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Kimi K2系列最新版本，强化编程与Agent集群能力，支持动态生成多个子Agent并行协作，已开源（发布时间在搜索窗口前，但为截至2026-06-05最新稳定版，广泛报道于6月初技术综述中）。</t>
+          <t>Kimi K2系列最新版本，强化编程与Agent集群能力，支持动态生成多个子Agent并行协作，已开源（发布时间在搜索窗口前，但为截至2026-06-05最新稳定版，广泛报道于6月初技术综述中）。 [重要性:高|月之暗面属于国内重点关注公司，Kimi K系列若为重要版本更新应高优先级关注。]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -954,10 +966,340 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→月之暗面/Moonshot AI; 官网→https://kimi.moonshot.cn/; 任务类型→通用对话/代码生成/智能体; 备注→Kimi K系列模型；强化编程与Agent能力；开源、多模态和子Agent协作能力需官方核实; 问题: 发布时间为2026-04-20，属于2026年内发布但明显超出本次2026-06-06窗口，应标注“窗口外”而非删除; 未能基于已知公开资料核实Kimi K2.6于2026-04-20官方发布; 类型标为“开源多模态智能体模型”需复核，尤其是开源状态和多模态能力; 备注中“动态生成多个子Agent并行协作”“截至2026-06-05最新稳定版”等表述需官方来源核实; 名称具备版本号，不属于产品泛称；因给定发布时间在2026年，按宽松保留原则不删除。</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HKGAI V3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>香港生成式人工智能研发中心（HKGAI）</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>香港首个本地研发的生产力级大模型V3版本，支持长上下文理解与多轮复杂推理，作为香港特区政府InnoHK创科平台重点成果发布。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HKGAI Super Agent（生产力级超级智能体）</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>香港生成式人工智能研发中心（HKGAI）</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>智能体</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>香港首个生产力级超级智能体，单次无干预稳定运行长达28小时，可端到端完成资料整理、推理分析、报告撰写及代码开发等复合任务。</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Google I/O 2026正式发布的极速工作流优化模型，支持100万tokens超长上下文，输出速度较上一代提升4倍，专为Agent编排与高频API调用设计。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Instant</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>GPT-5.5全量上线版本，聚焦可信度增强，医疗、法律等高敏感领域幻觉率下降52.5%，强调事实一致性与可验证输出。</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>码道（CodeArts）AI编程智能体</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>华为云</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>智能体（AI编程）</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>华为云全新商用AI编程智能体，聚焦全流程智能编码，支持需求理解、架构设计、代码生成、单元测试与部署建议，已于2026年5月30日正式商用。</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>心理健康测·评·析·预·训·辅一体化AI大模型系统</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>可家（成都）医学工程技术有限公司</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>垂直领域多模态大模型</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>国内首个面向青少年心理健康的全链路AI大模型系统，集成筛查评估、风险预测、认知训练与人工协同辅导能力。</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-08
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,14 +506,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>gemma-4-12B-it-qat-w4a16-ct</t>
+          <t>HKGAI V3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>香港生成式人工智能研发中心（HKGAI）</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,70 +521,58 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>12B</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/google/gemma-4-12B-it-qat-w4a16-ct</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace any-to-any</t>
+          <t>香港首个本地研发的生产力级大模型V3版本，支持长上下文理解与多轮复杂推理，作为香港特区政府InnoHK创科平台重点成果发布。 [重要性:低|其他机构发布的区域性大语言模型，具备一定本地化意义但尚未确认行业级突破。]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+          <t>2026-06-07 02:31</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>HuggingFace 已核实(google/gemma-4-12B-it-qat-w4a16-ct) · 参数量=13B · apache-2.0 · any-to-any</t>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(中置信)待人工确认 — 建议修正: 备注→香港本地研发；生产力级大语言模型；长上下文理解；多轮复杂推理; 任务类型→通用对话; 问题: 国内外字段疑似错误：香港生成式人工智能研发中心应归为国内/中国香港，而非国外; 官网缺失，需人工核实官方模型页面; 开闭源信息缺失; 发布时间为2026-06-03，位于追踪窗口前一周内，可保留但建议核实官方公告; 模型名称包含明确版本号V3，符合具体模型名称规范；但该模型的公开技术指标、参数规模、上下文长度等信息不足。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-08 02:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cosmos 3 (Super/Base/Tiny)</t>
+          <t>HKGAI Super Agent（生产力级超级智能体）</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>香港生成式人工智能研发中心（HKGAI）</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -596,29 +584,25 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>全模态物理AI基础模型</t>
+          <t>智能体</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://build.nvidia.com</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>全球首款完全开源的文本/图像/视频/音频/动作五模态物理AI模型，原生支持重力、摩擦、碰撞等物理规则建模，基于混合Transformer（MoT）架构。 [重要性:高|NVIDIA物理AI/世界模型若为重大版本更新，具备较高行业关注度和技术价值。]</t>
+          <t>香港首个生产力级超级智能体，单次无干预稳定运行长达28小时，可端到端完成资料整理、推理分析、报告撰写及代码开发等复合任务。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-07 02:31</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -628,56 +612,56 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://www.nvidia.com/en-us/ai/cosmos/; 任务类型→物理AI/世界模型; 备注→物理AI世界基础模型；多模态生成与理解；面向机器人与仿真场景；开源情况需核实; 问题: 模型名称包含多个变体Super/Base/Tiny，建议拆分为独立模型条目或明确主模型与子型号; 未能基于已知公开资料核实Cosmos 3于2026-06-01官方发布; 备注中“全球首款完全开源”“五模态”等表述需官方来源核实; 开源标注需复核，NVIDIA Cosmos系列可能存在开放权重、开放许可与完全开源的区别; 名称具备版本号，不属于产品泛称；如确为2026年6月发布，应保留。</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 该条目更像智能体产品/系统，不是具体模型名称+版本号; 国内外字段疑似错误：香港生成式人工智能研发中心应归为国内/中国香港，而非国外; 官网缺失，需人工核实官方页面; 开闭源信息缺失</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-06-08 02:33</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>码道（CodeArts）AI编程智能体</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>华为云</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>智能体（AI编程）</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://build.nvidia.com</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>千亿参数Dense架构LLM，MMLU-Pro达89.5分，支持INT4量化在RTX 5090上实时推理（首Token延迟低至180ms），面向消费级GPU优化。 [重要性:中|NVIDIA属于国外优秀关注公司，Nemotron若为新一代大模型更新值得关注。]</t>
+          <t>华为云全新商用AI编程智能体，聚焦全流程智能编码，支持需求理解、架构设计、代码生成、单元测试与部署建议，已于2026年5月30日正式商用。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-07 02:31</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -687,34 +671,38 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 官网→https://www.nvidia.com/en-us/ai-data-science/foundation-models/nemotron/; 任务类型→通用对话/推理; 备注→Nemotron系列大语言模型；面向推理与企业AI应用；参数规模、Benchmark与消费级GPU优化能力需官方核实; 问题: 未能基于已知公开资料核实Nemotron 3 Ultra于2026-06-01官方发布; “千亿参数Dense架构”“MMLU-Pro 89.5”“RTX 5090实时推理”等具体指标需官方来源核实; 名称具备版本/型号，不属于产品泛称; 建议人工核查NVIDIA官方博客、NVIDIA NIM/Build平台及技术报告。</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称为AI编程智能体/产品名称，未包含具体模型版本号或型号; 类型为智能体而非模型，若要收录需明确其底层模型名称和版本; 官网缺失，需人工核实官方产品页面; 开闭源信息缺失</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-06-08 02:33</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MiniMax M3</t>
+          <t>心理健康测·评·析·预·训·辅一体化AI大模型系统</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>可家（成都）医学工程技术有限公司</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
+          <t>垂直领域多模态大模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -722,17 +710,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>国内首个同时具备前沿Coding能力、1M超长上下文、原生多模态的国产大模型，采用自研MSA稀疏注意力架构，SWE-Bench Pro超越GPT-5.5。 [重要性:高|MiniMax属于国内重点关注公司，若M3为旗舰级多模态大模型则属于重大版本更新。]</t>
+          <t>国内首个面向青少年心理健康的全链路AI大模型系统，集成筛查评估、风险预测、认知训练与人工协同辅导能力。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-07 02:31</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -742,22 +730,26 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→MiniMax; 官网→https://www.minimax.io/; 任务类型→通用对话/多模态/代码生成; 备注→MiniMax系列多模态大模型；长上下文、代码能力与Agent能力需官方核实; 问题: 未能基于已知公开资料核实MiniMax M3于2026-06-01官方发布; “国内首个”“SWE-Bench Pro超越GPT-5.5”等强断言需官方或权威评测来源核实; 名称具备版本号，不属于产品泛称; 如官方确认发布时间为2026年，应保留；当前描述存在明显营销化和未核实Benchmark风险。</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5建议删除(中置信)待人工确认 — 建议删除：产品泛称无版本号; 名称为描述性系统名称，不是具体模型/产品名称+版本号; 国内外字段错误：公司位于成都，应归为国内; 更像垂直行业应用系统，不是明确的基础模型或具体模型版本; 官网缺失，需人工核实官方页面; 开闭源信息缺失</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-06-08 02:33</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Qwen3.7-Plus</t>
+          <t>Cosmos 3 (Super/Base/Tiny)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Alibaba (Tongyi Lab)</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -769,29 +761,25 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>多模态智能体模型</t>
+          <t>多模态物理AI基础模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://tongyi.aliyun.com/</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>主打‘看想做做验’一体化智能体能力，可连续11小时自主开发App，覆盖需求理解、代码生成、测试验证等全流程项目级任务。 [重要性:高|Qwen属于国内重点关注公司的核心模型系列，若为3.7代Plus更新则具备高关注价值。]</t>
+          <t>全球首款完全开源的全模态物理AI模型，原生支持文本/图像/视频/音频/动作五模态，精准复刻重力、摩擦、碰撞等物理规则，权重、代码、数据集全部开源至Hugging Face。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -801,7 +789,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→阿里巴巴/通义千问; 官网→https://qwenlm.github.io/; 任务类型→通用对话/多模态/智能体; 备注→Qwen系列Plus版本；面向通用对话、代码与智能体任务；具体长程Agent能力需官方核实; 问题: 公司名建议统一为“阿里巴巴/通义千问”; 原始数据中“国内外”标为国外，与阿里巴巴/通义千问不符，应为国内; 未能基于已知公开资料核实Qwen3.7-Plus于2026-06-02官方发布; 类型标为“多模态智能体模型”需复核，Plus版本可能是通用大模型而非专门智能体模型; 备注中“连续11小时自主开发App”等能力描述需官方评测或演示来源核实; 名称具备版本/型号，不属于产品泛称；建议核查Qwen官方博客、GitHub和模型卡。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -809,14 +797,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MAI-Code-1-Flash</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -828,7 +816,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>代码推理模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -836,17 +824,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>微软Build 2026发布的开源高级代码推理模型，专为复杂工程级代码生成与调试优化，支持多文件上下文协同推理。 [重要性:中|微软自研代码模型若属实，在代码生成领域具有较高应用价值，但不在重点关注公司清单内。]</t>
+          <t>千亿参数Dense架构LLM，128层Transformer，MMLU-Pro达89.5分，支持INT4量化在RTX 5090上实时推理，首Token延迟低至180ms，专为气隙部署与消费级GPU优化。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -856,7 +844,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Microsoft AI; 任务类型→代码生成/代码推理; 备注→代码推理模型；面向复杂工程级代码生成、调试与多文件上下文处理；开源情况需官方核实; 问题: 未能基于已知公开资料核实MAI-Code-1-Flash于2026-06-02官方发布; “Build 2026发布”“开源高级代码推理模型”等信息需微软官方公告核实; 开闭源标注缺失且备注称开源，建议补充并核实许可证; 名称具备版本/型号，不属于产品泛称; 建议核查Microsoft AI Blog、Build大会公告、Azure AI Foundry模型目录和GitHub。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -864,26 +852,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAI Thinking 1</t>
+          <t>MiniMax M3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>深度推理模型</t>
+          <t>多模态大语言模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -891,17 +879,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>微软自研的深度链式推理（Chain-of-Thought）增强模型，面向数学证明、逻辑规划与跨文档复杂决策任务。 [重要性:中|微软自研推理模型若属实属于重要厂商在推理方向的更新，具备中等以上关注价值。]</t>
+          <t>国内首个同时具备前沿Coding、1M超长上下文、原生多模态能力的大模型，自研MSA稀疏注意力架构，SWE-Bench Pro性能超越GPT-5.5与Gemini 3.1 Pro。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -911,7 +899,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→Microsoft AI; 任务类型→深度推理/通用对话; 备注→深度推理模型；面向数学、逻辑规划与复杂决策；具体推理机制和性能需官方核实; 问题: 未能基于已知公开资料核实MAI Thinking 1于2026-06-02官方发布; 模型命名是否应为“MAI-Thinking-1”或其他官方格式需复核; 备注中“深度链式推理增强”等技术描述需官方技术报告核实; 名称具备版本号，不属于产品泛称; 建议核查Microsoft AI官方博客、Azure AI Foundry及Build 2026发布资料。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -919,26 +907,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kimi K2.6</t>
+          <t>Qwen3.7-Plus</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Moonshot AI (月之暗面)</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>开源多模态智能体模型</t>
+          <t>多模态智能体模型</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -946,17 +934,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Kimi K2系列最新版本，强化编程与Agent集群能力，支持动态生成多个子Agent并行协作，已开源（发布时间在搜索窗口前，但为截至2026-06-05最新稳定版，广泛报道于6月初技术综述中）。 [重要性:高|月之暗面属于国内重点关注公司，Kimi K系列若为重要版本更新应高优先级关注。]</t>
+          <t>国产最强多模态智能体模型，支持‘看想做做验’一体化任务流，可连续11小时自主开发完整App，覆盖需求分析、编码、测试、部署全流程。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-06-06 02:02</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -966,7 +954,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）; ⚠️ GPT-5.5审核(低置信)待人工确认 — 建议修正: 公司→月之暗面/Moonshot AI; 官网→https://kimi.moonshot.cn/; 任务类型→通用对话/代码生成/智能体; 备注→Kimi K系列模型；强化编程与Agent能力；开源、多模态和子Agent协作能力需官方核实; 问题: 发布时间为2026-04-20，属于2026年内发布但明显超出本次2026-06-06窗口，应标注“窗口外”而非删除; 未能基于已知公开资料核实Kimi K2.6于2026-04-20官方发布; 类型标为“开源多模态智能体模型”需复核，尤其是开源状态和多模态能力; 备注中“动态生成多个子Agent并行协作”“截至2026-06-05最新稳定版”等表述需官方来源核实; 名称具备版本号，不属于产品泛称；因给定发布时间在2026年，按宽松保留原则不删除。</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -974,14 +962,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HKGAI V3</t>
+          <t>MAI-Thinking-1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>香港生成式人工智能研发中心（HKGAI）</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -993,7 +981,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>深度推理大语言模型</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1001,17 +989,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>香港首个本地研发的生产力级大模型V3版本，支持长上下文理解与多轮复杂推理，作为香港特区政府InnoHK创科平台重点成果发布。</t>
+          <t>微软Build 2026发布的旗舰推理模型，专注复杂逻辑链构建与长程规划，与Anthropic Claude Sonnet 4.6在编码基准上持平，已集成至Project Solara智能体操作系统。</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-06-07 02:31</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1029,14 +1017,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HKGAI Super Agent（生产力级超级智能体）</t>
+          <t>MAI-Code-1-Flash</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>香港生成式人工智能研发中心（HKGAI）</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1048,7 +1036,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>智能体</t>
+          <t>代码大语言模型</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1056,17 +1044,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>香港首个生产力级超级智能体，单次无干预稳定运行长达28小时，可端到端完成资料整理、推理分析、报告撰写及代码开发等复合任务。</t>
+          <t>50亿参数轻量级开源代码模型，专为GitHub生态优化，支持实时补全、单元测试生成与PR评论，推理延迟低于80ms（A100），已开放Hugging Face权重。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-06-07 02:31</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1084,14 +1072,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash</t>
+          <t>WorkBuddy 企业版</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>Tencent</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1103,7 +1091,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
+          <t>企业级效率智能体</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1111,17 +1099,17 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Google I/O 2026正式发布的极速工作流优化模型，支持100万tokens超长上下文，输出速度较上一代提升4倍，专为Agent编排与高频API调用设计。</t>
+          <t>腾讯云发布的面向中大型企业的AI工作台智能体，集成ClawPro引擎与TokenHub调度系统，支持跨OA/CRM/ERP自动执行审批、报表生成、会议纪要归档等复合任务。</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-06-07 02:31</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1139,14 +1127,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GPT-5.5 Instant</t>
+          <t>Efficiency Agent Toolkit</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Tencent</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1158,7 +1146,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>智能体工具集</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1166,17 +1154,17 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>GPT-5.5全量上线版本，聚焦可信度增强，医疗、法律等高敏感领域幻觉率下降52.5%，强调事实一致性与可验证输出。</t>
+          <t>包含QClaw、ima、元宝、腾讯文档AI插件等开箱即用智能体组件，支持个人与团队级自动化工作流编排，已在医疗、金融、零售等20+行业落地。</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-06-07 02:31</t>
+          <t>2026-06-08 02:35</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1190,116 +1178,6 @@
         </is>
       </c>
       <c r="Q13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>码道（CodeArts）AI编程智能体</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>华为云</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>智能体（AI编程）</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>华为云全新商用AI编程智能体，聚焦全流程智能编码，支持需求理解、架构设计、代码生成、单元测试与部署建议，已于2026年5月30日正式商用。</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>2026-06-07 02:31</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>心理健康测·评·析·预·训·辅一体化AI大模型系统</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>可家（成都）医学工程技术有限公司</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>垂直领域多模态大模型</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>国内首个面向青少年心理健康的全链路AI大模型系统，集成筛查评估、风险预测、认知训练与人工协同辅导能力。</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2026-06-07 02:31</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-10
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,7 +562,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-09 01:58</t>
+          <t>2026-06-10 02:11</t>
         </is>
       </c>
     </row>
@@ -621,21 +621,21 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-09 01:58</t>
+          <t>2026-06-10 02:11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>u2</t>
+          <t>Claude Fable 5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>云知声</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -643,42 +643,282 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>原生智能体大语言模型</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/claude-fable-5</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>面向个人、开发者与组织的通用大语言模型，具备自主拆解并执行100+步复杂工作流的能力，强调高智能密度与高token价值，在GPQA Diamond（87.9分）和GDPVal（72.5分）等权威评测中进入第一梯队。</t>
+          <t>1000k上下文；顶级编码能力；高端定价</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-09 01:58</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-06-10 02:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gemini 3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Google在WWDC26期间确认Gemini 3已集成至新版Siri，为苹果iOS 27提供底层AI能力，支持实时多模态推理与长上下文对话。</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-06-10 02:12</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>是</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DeepSeek V3.2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>深度求索/DeepSeek</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>面向企业级智能体场景优化的推理增强版本，在代码生成、数学推理和工具调用稳定性上显著提升，已通过国内多家银行与政务AI平台灰度部署。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-06-10 02:12</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GLM-5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>智谱AI</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>全新一代开源可商用大模型，支持1M上下文、原生多Agent协作协议，已在智谱「GLM OS」智能体平台同步上线。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-06-10 02:12</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kimi-Max</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>月之暗面/Kimi</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>长上下文多模态模型</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>专为医疗病理分析优化的Kimi系列新版本，支持200万token文档理解与显微图像-报告联合推理，已在合作三甲医院病理科启动临床验证。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-06-10 02:12</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-11
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-10 02:11</t>
+          <t>2026-06-11 02:34</t>
         </is>
       </c>
     </row>
@@ -621,21 +621,21 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-10 02:11</t>
+          <t>2026-06-11 02:34</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Claude Fable 5</t>
+          <t>DiffusionGemma 26B-A4B</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -645,10 +645,14 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>闭源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>25B</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>多模态</t>
@@ -656,7 +660,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>thinking</t>
+          <t>non-thinking</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -666,22 +670,22 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/claude-fable-5</t>
+          <t>https://llm-stats.com/models/diffusiongemma-26b-a4b-it</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1000k上下文；顶级编码能力；高端定价</t>
+          <t>MoE架构；25B参数；Apache 2.0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -691,26 +695,26 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜</t>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(google/DiffusionGemma 26B-A4B)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-06-10 02:11</t>
+          <t>2026-06-11 02:34</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gemini 3</t>
+          <t>diffusiongemma-26B-A4B-it-NVFP4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -718,66 +722,82 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>26B(A4B)</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/diffusiongemma-26B-A4B-it-NVFP4</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Google在WWDC26期间确认Gemini 3已集成至新版Siri，为苹果iOS 27提供底层AI能力，支持实时多模态推理与长上下文对话。</t>
+          <t>HuggingFace text-generation</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-10 02:12</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/diffusiongemma-26B-A4B-it-NVFP4)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-06-11 02:34</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DeepSeek V3.2</t>
+          <t>Fable5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>深度求索/DeepSeek</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>大语言模型（安全受限版）</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -785,17 +805,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>面向企业级智能体场景优化的推理增强版本，在代码生成、数学推理和工具调用稳定性上显著提升，已通过国内多家银行与政务AI平台灰度部署。</t>
+          <t>Anthropic发布的Mythos系列新版本，明确禁用网络安全与生物学相关能力，由Opus4.8处理敏感查询，旨在回应监管关切并配合IPO进程。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-10 02:12</t>
+          <t>2026-06-11 02:34</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -813,26 +833,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GLM-5</t>
+          <t>Mythos5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>智谱AI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>大语言模型（无防护开放版）</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -840,17 +860,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>全新一代开源可商用大模型，支持1M上下文、原生多Agent协作协议，已在智谱「GLM OS」智能体平台同步上线。</t>
+          <t>同步推出的Mythos5非限制版本，通过Project Glasswing计划向约200家组织开放，允许更自由的模型能力调用。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-10 02:12</t>
+          <t>2026-06-11 02:34</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -868,14 +888,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kimi-Max</t>
+          <t>Tabbit 1.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>月之暗面/Kimi</t>
+          <t>美团</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -887,7 +907,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>长上下文多模态模型</t>
+          <t>AI智能体浏览器</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -895,7 +915,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>专为医疗病理分析优化的Kimi系列新版本，支持200万token文档理解与显微图像-报告联合推理，已在合作三甲医院病理科启动临床验证。</t>
+          <t>国内首款浏览器形态AI原生入口，集成DeepSeek、LongCat、智谱GLM、Kimi等多模型，支持跨软件/跨网页自动执行复杂任务。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -905,7 +925,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-10 02:12</t>
+          <t>2026-06-11 02:34</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-14
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -812,6 +812,230 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>正式开放权重的超大规模模型，总参数约428B、激活参数23B，面向多模态理解与生成任务，支持本地部署与Agent集成。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-06-14 02:33</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>openPangu 2.0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>华为</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>开源大模型系列（含语言、视觉、科学计算等）</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>盘古大模型全新迭代版本，计划于6月30日起陆续开源核心组件，涵盖NLP、CV、气象、药物发现等多领域专用子模型。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-06-14 02:33</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PP-OCRv6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PaddleOCR（百度飞桨）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>光学字符识别模型</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>最新版端到端OCR模型，支持超轻量部署、多语言混合识别及复杂版式（如表格、手写、低质图像）鲁棒解析。</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-06-14 02:33</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MineExplorer</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>美团LongCat团队</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>智能体评测基准</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>首个面向开放世界环境的Agent评测基准，覆盖长程规划、工具调用、环境反馈适应与跨任务泛化能力评估。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-14 02:33</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-15
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kimi K2.7 Code</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Moonshot AI</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,64 +526,44 @@
           <t>国内</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1T</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>代码</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/kimi-k2.7-code</t>
-        </is>
-      </c>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>MoE架构；1T参数；262k上下文；MIT (modified)</t>
+          <t>正式开放权重的超大规模模型，总参数约428B、激活参数23B，面向多模态理解与生成任务，支持本地部署与Agent集成。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14 02:33</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>是</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜 · HuggingFace 需登录(moonshot-ai/Kimi K2.7 Code)</t>
+          <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-13 02:09</t>
+          <t>2026-06-15 02:41</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -591,26 +571,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BAAI Cardiac Agent v1.0</t>
+          <t>openPangu 2.0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>智源研究院</t>
+          <t>华为</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>医疗诊断智能体</t>
+          <t>开源大模型系列（含语言、视觉、科学计算等）</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -618,17 +598,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>首个面向心脏磁共振多模态数据的辅助诊断智能体，由智源研究院与安贞医院联合研发，诊断精度达顶尖心血管医生水平。</t>
+          <t>盘古大模型全新迭代版本，计划于6月30日起陆续开源核心组件，涵盖NLP、CV、气象、药物发现等多领域专用子模型。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-13 02:10</t>
+          <t>2026-06-14 02:33</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -641,50 +621,58 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-06-15 02:41</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AREX v1.0</t>
+          <t>PP-OCRv6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>智源研究院</t>
+          <t>PaddleOCR（百度飞桨）</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>科学发现智能体</t>
+          <t>光学字符识别模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://github.com/PaddlePaddle/PaddleOCR</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>面向基础科研全流程的自主研究智能体，支持文献调研、实验设计、结果论证与论文撰写，推动AI驱动的自主科学发现。</t>
+          <t>最新版端到端OCR模型，支持超轻量部署、多语言混合识别及复杂版式（如表格、手写、低质图像）鲁棒解析。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-13 02:10</t>
+          <t>2026-06-14 02:33</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -697,32 +685,36 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-06-15 02:41</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SoulAgent v1.0</t>
+          <t>MineExplorer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>智源研究院</t>
+          <t>美团LongCat团队</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>个人专属智能体</t>
+          <t>智能体评测基准</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -730,17 +722,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>采用自研轻量架构的个人数字分身智能体，Token成本节省30%，资源占用降低80%，支持小程序端即时交互。</t>
+          <t>首个面向开放世界环境的Agent评测基准，覆盖长程规划、工具调用、环境反馈适应与跨任务泛化能力评估。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-13 02:10</t>
+          <t>2026-06-14 02:33</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -753,32 +745,36 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-06-15 02:41</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RiskGuard Bio-Agent v1.0</t>
+          <t>GLM-5.2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>智源研究院</t>
+          <t>智谱AI (Z.ai)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>AI安全智能体</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -786,17 +782,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>面向生物安全的风险发现智能体，通过主动模拟攻击者行为，识别有害蛋白序列设计等环节的脆弱性，实现生物风险‘事前演练’防控。</t>
+          <t>旗舰开源大模型，支持1M上下文、High/Max双档思考强度，官方称其为‘迄今能力最强的开源模型’，API及MIT协议开源版本计划下周上线。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-13 02:10</t>
+          <t>2026-06-15 02:42</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -815,14 +811,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>ZCode 3.0.0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>智谱AI (Z.ai)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -834,7 +830,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
+          <t>智能体开发框架</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -842,17 +838,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>正式开放权重的超大规模模型，总参数约428B、激活参数23B，面向多模态理解与生成任务，支持本地部署与Agent集成。</t>
+          <t>全新自研Agent内核编程工具，深度适配GLM-5.2，新增分组式任务工作区、Zread智能知识库与可视化Git分支图谱，全面替代第三方Agent框架。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-14 02:33</t>
+          <t>2026-06-15 02:42</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -871,26 +867,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>openPangu 2.0</t>
+          <t>ZONOS2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>华为</t>
+          <t>Zyphra</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>开源大模型系列（含语言、视觉、科学计算等）</t>
+          <t>文本到语音（TTS）模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -898,17 +894,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>盘古大模型全新迭代版本，计划于6月30日起陆续开源核心组件，涵盖NLP、CV、气象、药物发现等多领域专用子模型。</t>
+          <t>开源高质量TTS模型，支持多语种、高保真语音合成，强调低延迟与端侧部署友好性。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-14 02:33</t>
+          <t>2026-06-15 02:42</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -923,118 +919,6 @@
       </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PP-OCRv6</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>PaddleOCR（百度飞桨）</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>光学字符识别模型</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>最新版端到端OCR模型，支持超轻量部署、多语言混合识别及复杂版式（如表格、手写、低质图像）鲁棒解析。</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-06-14 02:33</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MineExplorer</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>美团LongCat团队</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>智能体评测基准</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>首个面向开放世界环境的Agent评测基准，覆盖长程规划、工具调用、环境反馈适应与跨任务泛化能力评估。</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-06-14 02:33</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-16
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -920,6 +920,1350 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>速度提升2.5倍，代码缺陷比上一代减少4倍，代理推理成本降61%</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Grok-Imagine-Video-1.5-Preview</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SpaceXAI</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>视频生成模型</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>面向长时序、高保真视频生成的预览版模型，已开放API</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Qwen-VLA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>统一视觉语言动作模型</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>首个支持端到端视觉-语言-动作联合建模的通用具身智能基础模型</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Qwen3.7-Plus</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>多模态智能体模型</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>面向复杂任务编排与工具调用优化的多模态智能体模型，强化工作流闭环能力</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Project Eden (Preview)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VAST</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>多人多智能体世界模型</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>支持多智能体协同仿真、物理交互与社会规则建模的世界模型预览版</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mellum2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>JetBrains</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>代码模型</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>12B MoE架构低延迟代码补全与推理模型，专为IDE实时交互优化</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Holo3.1 系列</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>H Company</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>端侧优化模型</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>面向手机/AR眼镜等终端设备的轻量化多模态模型系列，支持本地化智能体运行</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ideogram 4.0</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ideogram</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>文生图模型</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>9.3B参数开源文生图模型，显著提升文本忠实度与复杂构图能力</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Reve 2.0</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Reve</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>图像生成与编辑模型</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>支持4K分辨率生成与像素级精细化编辑的顶级图像模型</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GPT-Rosalind (升级版)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>生命科学专用大模型</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>面向蛋白质结构预测、基因序列分析与药物分子设计深度优化的GPT系列专业模型</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Nex-N2-Pro</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Nex-AGI</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>旗舰开源大模型</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>对标顶级商用模型的开源大语言模型，被证实为Rio 3.5底层技术主干之一</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Bernini</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>字节跳动</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>视频生成编辑统一框架</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>支持生成、剪辑、重绘、运镜控制的一体化开源视频AI框架</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Higgs Audio v3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Boson AI</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>语音合成模型</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>多语种TTS模型，支持情感可控、零样本克隆与实时流式合成</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Magenta RealTime 2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Google Magenta</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>音乐生成模型</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>低延迟实时音乐生成模型，支持毫秒级响应与多乐器协同即兴</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Nemotron 3.5</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>多模态内容安全审核模型</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>开源多模态安全模型，支持图文音视频跨模态有害内容识别与细粒度归因</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HKGAI V3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>香港HKGAI</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>本地化智能体大模型</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>面向粤语及港澳场景深度优化的智能体模型，强化政务、金融、教育垂直能力</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Gemma 4 12B</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>轻量多模态模型</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>开源12B参数多模态模型，支持原生音频输入，适配普通终端设备运行</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Gemma 4 QAT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>量化模型</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Gemma 4系列移动端QAT量化权重，模型压缩至1GB以内</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>dots.tts</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>小红书</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>端到端TTS模型</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>20亿参数开源端到端中文TTS模型，支持高自然度与风格迁移</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Riverflow 2.5</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OpenRouter</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>自定义图像模型</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>支持用户上传LoRA/ControlNet配置的可定制文生图模型，限时免费开放</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MisoTTS 8B</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Miso Labs</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>情感TTS模型</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>8B参数开源情感语音合成模型，支持细粒度情绪强度与角色风格控制</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BLS-Mini-Code-1.0</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>编程专用模型</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>早期测试版轻量级编程模型，聚焦Python/TypeScript代码补全与单元测试生成</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Harness-1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>高校团队</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>搜索智能体</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>20B高性能开源搜索智能体，支持多跳检索、结果验证与自主信息溯源</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>OpenClaw 6.6</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OpenClaw社区</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>AI智能体框架</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>开源智能体框架新版本，实现‘目标→规划→工具调用→自动执行’闭环，支持邮件整理、日程管理等真实工作流</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:41</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-17
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,44 +511,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Grok-Imagine-Video-1.5-Preview</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
+          <t>视频生成模型</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://docs.x.ai/developers/models/grok-imagine-video-1.5-preview</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>正式开放权重的超大规模模型，总参数约428B、激活参数23B，面向多模态理解与生成任务，支持本地部署与Agent集成。</t>
+          <t>面向长时序、高保真视频生成的预览版模型，已开放API</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-14 02:33</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -563,7 +567,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-15 02:41</t>
+          <t>2026-06-17 02:37</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -571,14 +575,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>openPangu 2.0</t>
+          <t>Qwen-VLA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>华为</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -590,7 +594,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>开源大模型系列（含语言、视觉、科学计算等）</t>
+          <t>统一视觉语言动作模型</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -598,17 +602,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>盘古大模型全新迭代版本，计划于6月30日起陆续开源核心组件，涵盖NLP、CV、气象、药物发现等多领域专用子模型。</t>
+          <t>首个支持端到端视觉-语言-动作联合建模的通用具身智能基础模型</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-14 02:33</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -623,7 +627,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-15 02:41</t>
+          <t>2026-06-17 02:37</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -631,48 +635,44 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PP-OCRv6</t>
+          <t>Project Eden (Preview)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PaddleOCR（百度飞桨）</t>
+          <t>VAST</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>光学字符识别模型</t>
+          <t>多人多智能体世界模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://github.com/PaddlePaddle/PaddleOCR</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>最新版端到端OCR模型，支持超轻量部署、多语言混合识别及复杂版式（如表格、手写、低质图像）鲁棒解析。</t>
+          <t>支持多智能体协同仿真、物理交互与社会规则建模的世界模型预览版</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-14 02:33</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-06-15 02:41</t>
+          <t>2026-06-17 02:37</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -695,26 +695,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MineExplorer</t>
+          <t>Mellum2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>美团LongCat团队</t>
+          <t>JetBrains</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>智能体评测基准</t>
+          <t>代码模型</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -722,17 +722,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>首个面向开放世界环境的Agent评测基准，覆盖长程规划、工具调用、环境反馈适应与跨任务泛化能力评估。</t>
+          <t>12B MoE架构低延迟代码补全与推理模型，专为IDE实时交互优化</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-14 02:33</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-06-15 02:41</t>
+          <t>2026-06-17 02:37</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
@@ -755,26 +755,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GLM-5.2</t>
+          <t>Holo3.1 系列</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>智谱AI (Z.ai)</t>
+          <t>H Company</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>端侧优化模型</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -782,17 +782,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>旗舰开源大模型，支持1M上下文、High/Max双档思考强度，官方称其为‘迄今能力最强的开源模型’，API及MIT协议开源版本计划下周上线。</t>
+          <t>面向手机/AR眼镜等终端设备的轻量化多模态模型系列，支持本地化智能体运行</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-15 02:42</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -805,32 +805,36 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ZCode 3.0.0</t>
+          <t>Ideogram 4.0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>智谱AI (Z.ai)</t>
+          <t>Ideogram</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>智能体开发框架</t>
+          <t>文生图模型</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -838,17 +842,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>全新自研Agent内核编程工具，深度适配GLM-5.2，新增分组式任务工作区、Zread智能知识库与可视化Git分支图谱，全面替代第三方Agent框架。</t>
+          <t>9.3B参数开源文生图模型，显著提升文本忠实度与复杂构图能力</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-15 02:42</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -861,20 +865,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ZONOS2</t>
+          <t>Reve 2.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Zyphra</t>
+          <t>Reve</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -886,25 +894,29 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>文本到语音（TTS）模型</t>
+          <t>图像生成与编辑模型</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://reve.com</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>开源高质量TTS模型，支持多语种、高保真语音合成，强调低延迟与端侧部署友好性。</t>
+          <t>支持4K分辨率生成与像素级精细化编辑的顶级图像模型</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-15 02:42</t>
+          <t>2026-06-16 02:41</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -917,20 +929,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Claude Opus 4.8</t>
+          <t>GPT-Rosalind (升级版)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -942,7 +958,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>生命科学专用大模型</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -950,12 +966,12 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>速度提升2.5倍，代码缺陷比上一代减少4倍，代理推理成本降61%</t>
+          <t>面向蛋白质结构预测、基因序列分析与药物分子设计深度优化的GPT系列专业模型</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -973,20 +989,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Grok-Imagine-Video-1.5-Preview</t>
+          <t>Nex-N2-Pro</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Nex-AGI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -998,7 +1018,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>视频生成模型</t>
+          <t>旗舰开源大模型</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1006,12 +1026,12 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>面向长时序、高保真视频生成的预览版模型，已开放API</t>
+          <t>对标顶级商用模型的开源大语言模型，被证实为Rio 3.5底层技术主干之一</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1029,20 +1049,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Qwen-VLA</t>
+          <t>Bernini</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>字节跳动</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1054,20 +1078,24 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>统一视觉语言动作模型</t>
+          <t>视频生成编辑统一框架</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://bernini-ai.github.io/</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>首个支持端到端视觉-语言-动作联合建模的通用具身智能基础模型</t>
+          <t>支持生成、剪辑、重绘、运镜控制的一体化开源视频AI框架</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1085,32 +1113,36 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Qwen3.7-Plus</t>
+          <t>Higgs Audio v3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>Boson AI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>多模态智能体模型</t>
+          <t>语音合成模型</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1118,12 +1150,12 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>面向复杂任务编排与工具调用优化的多模态智能体模型，强化工作流闭环能力</t>
+          <t>多语种TTS模型，支持情感可控、零样本克隆与实时流式合成</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1141,20 +1173,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Project Eden (Preview)</t>
+          <t>Magenta RealTime 2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>VAST</t>
+          <t>Google Magenta</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1166,20 +1202,24 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>多人多智能体世界模型</t>
+          <t>音乐生成模型</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://github.com/magenta/magenta-realtime</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>支持多智能体协同仿真、物理交互与社会规则建模的世界模型预览版</t>
+          <t>低延迟实时音乐生成模型，支持毫秒级响应与多乐器协同即兴</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1197,20 +1237,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mellum2</t>
+          <t>Nemotron 3.5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>JetBrains</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1222,7 +1266,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>代码模型</t>
+          <t>多模态内容安全审核模型</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1230,12 +1274,12 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>12B MoE架构低延迟代码补全与推理模型，专为IDE实时交互优化</t>
+          <t>开源多模态安全模型，支持图文音视频跨模态有害内容识别与细粒度归因</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1253,20 +1297,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Holo3.1 系列</t>
+          <t>dots.tts</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>H Company</t>
+          <t>小红书</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1278,20 +1326,24 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>端侧优化模型</t>
+          <t>端到端TTS模型</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://github.com/rednote-hilab/dots.tts</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>面向手机/AR眼镜等终端设备的轻量化多模态模型系列，支持本地化智能体运行</t>
+          <t>20亿参数开源端到端中文TTS模型，支持高自然度与风格迁移</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1309,20 +1361,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ideogram 4.0</t>
+          <t>Riverflow 2.5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ideogram</t>
+          <t>OpenRouter</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1334,7 +1390,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>文生图模型</t>
+          <t>自定义图像模型</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1342,12 +1398,12 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>9.3B参数开源文生图模型，显著提升文本忠实度与复杂构图能力</t>
+          <t>支持用户上传LoRA/ControlNet配置的可定制文生图模型，限时免费开放</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1365,20 +1421,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Reve 2.0</t>
+          <t>MisoTTS 8B</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Reve</t>
+          <t>Miso Labs</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1390,7 +1450,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>图像生成与编辑模型</t>
+          <t>情感TTS模型</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1398,12 +1458,12 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>支持4K分辨率生成与像素级精细化编辑的顶级图像模型</t>
+          <t>8B参数开源情感语音合成模型，支持细粒度情绪强度与角色风格控制</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1421,20 +1481,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GPT-Rosalind (升级版)</t>
+          <t>BLS-Mini-Code-1.0</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Cohere</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1446,20 +1510,24 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>生命科学专用大模型</t>
+          <t>编程专用模型</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://docs.cohere.com/docs/north-mini-code-1.0</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>面向蛋白质结构预测、基因序列分析与药物分子设计深度优化的GPT系列专业模型</t>
+          <t>早期测试版轻量级编程模型，聚焦Python/TypeScript代码补全与单元测试生成</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1477,20 +1545,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nex-N2-Pro</t>
+          <t>Harness-1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nex-AGI</t>
+          <t>高校团队</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1502,7 +1574,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>旗舰开源大模型</t>
+          <t>搜索智能体</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1510,12 +1582,12 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>对标顶级商用模型的开源大语言模型，被证实为Rio 3.5底层技术主干之一</t>
+          <t>20B高性能开源搜索智能体，支持多跳检索、结果验证与自主信息溯源</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1533,45 +1605,53 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bernini</t>
+          <t>OpenClaw 6.6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>字节跳动</t>
+          <t>OpenClaw社区</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>视频生成编辑统一框架</t>
+          <t>AI智能体框架</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://github.com/openclaw/openclaw</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>支持生成、剪辑、重绘、运镜控制的一体化开源视频AI框架</t>
+          <t>开源智能体框架新版本，实现‘目标→规划→工具调用→自动执行’闭环，支持邮件整理、日程管理等真实工作流</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1589,20 +1669,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:37</t>
+        </is>
+      </c>
       <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Higgs Audio v3</t>
+          <t>Anthropic Claude Fable 5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Boson AI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1614,7 +1698,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>语音合成模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1622,17 +1706,17 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>多语种TTS模型，支持情感可控、零样本克隆与实时流式合成</t>
+          <t>Anthropic发布的最强公开模型，发布仅3天后因美国紧急出口管制被全面关停，成为首个被列为‘国家安全资产’而遭强制召回的前沿AI模型。</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-06-16 02:41</t>
+          <t>2026-06-17 02:39</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1651,14 +1735,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Magenta RealTime 2</t>
+          <t>Anthropic Claude Mythos 5</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Google Magenta</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1670,7 +1754,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>音乐生成模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -1678,17 +1762,17 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>低延迟实时音乐生成模型，支持毫秒级响应与多乐器协同即兴</t>
+          <t>与Fable 5同期发布的高推理能力模型，同样于发布三日内被美国政府出口管制令波及，全球服务暂停。</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-06-16 02:41</t>
+          <t>2026-06-17 02:39</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1707,26 +1791,26 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Nemotron 3.5</t>
+          <t>智谱GLM-5.2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>智谱AI</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>多模态内容安全审核模型</t>
+          <t>大语言模型</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1734,17 +1818,17 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>开源多模态安全模型，支持图文音视频跨模态有害内容识别与细粒度归因</t>
+          <t>全量用户开放的最新版本GLM系列模型，支持多轮复杂推理与长上下文理解，将于下周开源API，作为对Claude Fable 5被禁的国产替代响应。</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-06-16 02:41</t>
+          <t>2026-06-17 02:39</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -1763,14 +1847,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HKGAI V3</t>
+          <t>星源智 ω-EVA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>香港HKGAI</t>
+          <t>星源智</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1782,7 +1866,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>本地化智能体大模型</t>
+          <t>具身智能世界模型</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1790,17 +1874,17 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>面向粤语及港澳场景深度优化的智能体模型，强化政务、金融、教育垂直能力</t>
+          <t>业界首个进入‘预演-验证-行动’决策闭环的世界模型，专为机器人物理交互设计，支持后果预判与自我修正。</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-06-16 02:41</t>
+          <t>2026-06-17 02:39</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -1819,14 +1903,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gemma 4 12B</t>
+          <t>理想汽车马赫M100具身智能模型</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>理想汽车</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1838,7 +1922,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>轻量多模态模型</t>
+          <t>具身智能模型</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -1846,17 +1930,17 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>开源12B参数多模态模型，支持原生音频输入，适配普通终端设备运行</t>
+          <t>面向‘具身智能汽车’场景自研的动态数据流AI模型，融合车控、驾乘交互、生活服务与职业司机辅助能力。</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-06-16 02:41</t>
+          <t>2026-06-17 02:39</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -1875,14 +1959,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Gemma 4 QAT</t>
+          <t>Rio-3.5-Open-397B</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>IplanRIO（巴西里约市政府）</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1894,7 +1978,7 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>量化模型</t>
+          <t>开源大语言模型（后证实为套壳）</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -1902,17 +1986,17 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Gemma 4系列移动端QAT量化权重，模型压缩至1GB以内</t>
+          <t>宣称由巴西官方发布的拉美首个SOTA级开源大模型，实为阿里通义千问Qwen3.5与Nex N2 Pro权重混合版本，发布24小时内公开致歉并下架。</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-06-16 02:41</t>
+          <t>2026-06-17 02:39</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -1927,342 +2011,6 @@
       </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>dots.tts</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>小红书</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>端到端TTS模型</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>20亿参数开源端到端中文TTS模型，支持高自然度与风格迁移</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>2026-06-16 02:41</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Riverflow 2.5</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>OpenRouter</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>自定义图像模型</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>支持用户上传LoRA/ControlNet配置的可定制文生图模型，限时免费开放</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>2026-06-16 02:41</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>MisoTTS 8B</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Miso Labs</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>情感TTS模型</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>8B参数开源情感语音合成模型，支持细粒度情绪强度与角色风格控制</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>2026-06-16 02:41</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>BLS-Mini-Code-1.0</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Cohere</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>编程专用模型</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>早期测试版轻量级编程模型，聚焦Python/TypeScript代码补全与单元测试生成</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>2026-06-16 02:41</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Harness-1</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>高校团队</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>搜索智能体</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>20B高性能开源搜索智能体，支持多跳检索、结果验证与自主信息溯源</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>2026-06-16 02:41</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>OpenClaw 6.6</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>OpenClaw社区</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>AI智能体框架</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>开源智能体框架新版本，实现‘目标→规划→工具调用→自动执行’闭环，支持邮件整理、日程管理等真实工作流</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>2026-06-16 02:41</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-18
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -839,7 +839,11 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://ideogram.ai</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>9.3B参数开源文生图模型，显著提升文本忠实度与复杂构图能力</t>
@@ -1147,7 +1151,11 @@
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://boson.ai</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>多语种TTS模型，支持情感可控、零样本克隆与实时流式合成</t>
@@ -1271,7 +1279,11 @@
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://www.nvidia.com/en-us/ai-data-science/generative-ai/nemotron/</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>开源多模态安全模型，支持图文音视频跨模态有害内容识别与细粒度归因</t>
@@ -1395,7 +1407,11 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://openrouter.ai</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>支持用户上传LoRA/ControlNet配置的可定制文生图模型，限时免费开放</t>
@@ -1703,7 +1719,11 @@
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/news/claude-fable-5-mythos-5</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>Anthropic发布的最强公开模型，发布仅3天后因美国紧急出口管制被全面关停，成为首个被列为‘国家安全资产’而遭强制召回的前沿AI模型。</t>
@@ -1759,7 +1779,11 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/news/claude-fable-5-mythos-5</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>与Fable 5同期发布的高推理能力模型，同样于发布三日内被美国政府出口管制令波及，全球服务暂停。</t>
@@ -1983,7 +2007,11 @@
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/prefeitura-rio/Rio-3.5-Open-397B</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>宣称由巴西官方发布的拉美首个SOTA级开源大模型，实为阿里通义千问Qwen3.5与Nex N2 Pro权重混合版本，发布24小时内公开致歉并下架。</t>
@@ -2011,6 +2039,398 @@
       </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>MiniMax于6月1日发布的旗舰模型，具备原生多模态、150万Token超长上下文及高阶智能体能力，编程评测成绩超越GPT-5.5</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GPT-5.6</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>OpenAI于6月17日推出的GPT系列新版本，显著提升编码效率与智能体工作流能力</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Gemini Omni</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>多模态大模型</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>谷歌在Android 17正式版中深度集成的多模态大模型，支持跨模态理解与生成，面向Pixel设备优化部署</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Lyria 3</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>音乐生成模型</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>谷歌发布的第三代端到端音乐生成模型，支持长时序、风格可控、实时交互式创作，集成于Pixel 10a及Wear OS 7</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Gemma 4 12B</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>轻量多模态模型</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>开源的12B参数多模态模型，支持原生音频输入，适配普通终端设备运行，大幅降低AI开发门槛</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>京东视觉语言实时交互模型（未命名）</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>京东</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>视觉语言智能体</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>支持摄像头/直播流/监控流+语音I/O的实时流式交互模型，计划开源权重、数据、训练方法及完整系统</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>WorkBuddy</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>腾讯</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>AI智能体</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>腾讯桌面办公效率智能体，已接入微信支付AI专属卡，支持任务自动化与跨应用协同</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:41</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-20
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,7 +767,11 @@
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://ai.google.dev/</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>谷歌I/O 2026推出的极速版模型，专为低延迟智能体服务设计，支撑全天候个人智能体Spark实时响应</t>
@@ -852,6 +856,230 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AstraBrain-WBC 0.5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>银河通用机器人</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>人形机器人通用小脑基础模型</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>全球首个人形机器人通用小脑GPT基础模型，基于2万小时人类动作数据训练，8040万参数，支持全身实时运动控制</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:12</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Qwen-RobotWorld</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>具身智能世界模型</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>千问具身智能大模型系列中的世界模型大脑组件，在WorldModelBench评测中总分8.99（开源模型第一），专注物理因果推演与仿真</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:12</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HappyOyster 1.0</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>阿里巴巴/通义</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>交互式世界模型</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>面向交互式内容生成的世界模型，支持动态环境建模与多轮具身交互推演</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:12</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Spark</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Google/DeepMind</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>个人智能体</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>谷歌I/O发布的全天候主动式个人智能体，重构搜索引擎从被动查询到主动服务范式</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:12</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-21
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lyria 3</t>
+          <t>AstraBrain-WBC 0.5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>银河通用机器人</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -530,7 +530,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>音乐生成模型</t>
+          <t>人形机器人通用小脑基础模型</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -538,17 +538,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>谷歌发布的第三代端到端音乐生成模型，支持长时序、风格可控、实时交互式创作，集成于Pixel 10a及Wear OS 7</t>
+          <t>全球首个人形机器人通用小脑GPT基础模型，基于2万小时人类动作数据训练，8040万参数，支持全身实时运动控制</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-18 02:41</t>
+          <t>2026-06-20 02:12</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-19 02:50</t>
+          <t>2026-06-21 02:35</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -571,14 +571,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>京东视觉语言实时交互模型（未命名）</t>
+          <t>Qwen-RobotWorld</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>京东</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -590,7 +590,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>视觉语言智能体</t>
+          <t>具身智能世界模型</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -598,17 +598,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>支持摄像头/直播流/监控流+语音I/O的实时流式交互模型，计划开源权重、数据、训练方法及完整系统</t>
+          <t>千问具身智能大模型系列中的世界模型大脑组件，在WorldModelBench评测中总分8.99（开源模型第一），专注物理因果推演与仿真</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-18 02:41</t>
+          <t>2026-06-20 02:12</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-19 02:50</t>
+          <t>2026-06-21 02:35</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -631,14 +631,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>HappyOyster 1.0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>阿里巴巴/通义</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -650,25 +650,29 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
+          <t>交互式世界模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.happyoyster.cn</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>MiniMax于6月1日发布的旗舰原生多模态模型，支持150万Token超长上下文、高阶智能体能力，编程评测成绩超越GPT-5.5</t>
+          <t>面向交互式内容生成的世界模型，支持动态环境建模与多轮具身交互推演</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-19 02:51</t>
+          <t>2026-06-20 02:12</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -681,20 +685,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-06-21 02:35</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GPT-5.6</t>
+          <t>Spark</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google/DeepMind</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -706,7 +714,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>大语言模型</t>
+          <t>个人智能体</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -714,17 +722,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>OpenAI于2026年6月正式发布的GPT-5.6版本，重点优化编码效率与智能体工作流能力，强化企业级权限管控与语音交互支持</t>
+          <t>谷歌I/O发布的全天候主动式个人智能体，重构搜索引擎从被动查询到主动服务范式</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-19 02:51</t>
+          <t>2026-06-20 02:12</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -737,20 +745,24 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-06-21 02:35</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash</t>
+          <t>&gt;&lt;former (v1.0)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>MIT &amp; MIT-IBM Watson AI Lab</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -762,29 +774,25 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>轻量级多模态大语言模型</t>
+          <t>neural network architecture</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://ai.google.dev/</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>谷歌I/O 2026推出的极速版模型，专为低延迟智能体服务设计，支撑全天候个人智能体Spark实时响应</t>
+          <t>一种颠覆性‘中间瘦两头胖’结构的新型Transformer变体，挑战传统等宽层设计，旨在提升能效比与推理效率。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-19 02:51</t>
+          <t>2026-06-21 02:36</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -803,14 +811,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gemma 4 12B</t>
+          <t>Vera CPU (first-generation)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -822,7 +830,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>开源轻量多模态模型</t>
+          <t>AI-optimized CPU</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -830,17 +838,17 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>谷歌同步开源的12B参数多模态模型，支持原生音频输入，可在普通终端设备本地运行，显著降低AI开发与部署门槛</t>
+          <t>英伟达首款独立CPU产品线，专为AI智能体时代token级低延迟调度与多智能体协同推理设计，已交付OpenAI和Anthropic首批试用。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-06-19 02:51</t>
+          <t>2026-06-21 02:36</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -859,14 +867,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AstraBrain-WBC 0.5</t>
+          <t>Mythos (unreleased public version, but newly designated as 'Frontier Model' under US executive order)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>银河通用机器人</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -878,7 +886,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>人形机器人通用小脑基础模型</t>
+          <t>frontier multimodal LLM</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -886,17 +894,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>全球首个人形机器人通用小脑GPT基础模型，基于2万小时人类动作数据训练，8040万参数，支持全身实时运动控制</t>
+          <t>虽未正式对外发布新版本，但特朗普6月2日签署行政令明确将Anthropic Mythos列为首批纳入联邦高风险模型评估体系的‘前沿模型’，标志其完成内部迭代并进入监管认定阶段。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-06-20 02:12</t>
+          <t>2026-06-21 02:36</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -911,174 +919,6 @@
       </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Qwen-RobotWorld</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>阿里巴巴/通义</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>具身智能世界模型</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>千问具身智能大模型系列中的世界模型大脑组件，在WorldModelBench评测中总分8.99（开源模型第一），专注物理因果推演与仿真</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-06-20 02:12</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>HappyOyster 1.0</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>阿里巴巴/通义</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>交互式世界模型</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>面向交互式内容生成的世界模型，支持动态环境建模与多轮具身交互推演</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-06-20 02:12</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Spark</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Google/DeepMind</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>个人智能体</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>谷歌I/O发布的全天候主动式个人智能体，重构搜索引擎从被动查询到主动服务范式</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2026-06-20 02:12</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-22
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -835,7 +835,11 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/nvidia-announces-next-generation-ai-platform-rubin-vera-and-nvlink-6</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>英伟达首款独立CPU产品线，专为AI智能体时代token级低延迟调度与多智能体协同推理设计，已交付OpenAI和Anthropic首批试用。</t>
@@ -920,6 +924,286 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>OpenAI Personal AGI Assistant (v0.1 prototype)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>智能体（Personal AGI Assistant）</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>OpenAI发布首个面向个人用户的AGI助手原型愿景，聚焦于日常任务、工作、学习与探索的高能力自主智能体，非开源模型，处于内部研究加速阶段规划中。</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:40</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>微信小微（测试版）</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>腾讯</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>原生AI智能体</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>腾讯在微信主界面上线小范围灰度测试的原生AI助手‘小微’，支持文字/语音交互操控微信原生功能，融合腾讯自研及优质开源多模型技术栈。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:40</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>智谱AI</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>大语言模型</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>智谱AI正式开源GLM-5.2，为GLM-5系列最新迭代版本，强化长上下文理解、工具调用与多步推理能力，支持1M tokens上下文与结构化输出。</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:40</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kimi-Max v2026.06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>月之暗面</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>多模态大语言模型</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>月之暗面发布Kimi-Max新版本，集成实时视频理解、高精度文档解析与跨模态推理能力，专为专业办公与科研场景优化，已接入部分企业API平台。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:40</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>混元T3-Agent</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>腾讯</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>智能体框架</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>腾讯混元团队发布轻量化智能体运行时框架T3-Agent，支持低延迟本地化部署、多工具自动编排与微信生态深度协同，面向小程序与企业服务场景开放内测。</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:40</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-23
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AstraBrain-WBC 0.5</t>
+          <t>OpenAI Personal AGI Assistant (v0.1 prototype)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>银河通用机器人</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -530,7 +530,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>人形机器人通用小脑基础模型</t>
+          <t>智能体（Personal AGI Assistant）</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -538,17 +538,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>全球首个人形机器人通用小脑GPT基础模型，基于2万小时人类动作数据训练，8040万参数，支持全身实时运动控制</t>
+          <t>OpenAI发布首个面向个人用户的AGI助手原型愿景，聚焦于日常任务、工作、学习与探索的高能力自主智能体，非开源模型，处于内部研究加速阶段规划中。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-20 02:12</t>
+          <t>2026-06-22 02:40</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-21 02:35</t>
+          <t>2026-06-23 02:05</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -571,14 +571,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Qwen-RobotWorld</t>
+          <t>微信小微（测试版）</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>腾讯</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -590,7 +590,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>具身智能世界模型</t>
+          <t>原生AI智能体</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -598,17 +598,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>千问具身智能大模型系列中的世界模型大脑组件，在WorldModelBench评测中总分8.99（开源模型第一），专注物理因果推演与仿真</t>
+          <t>腾讯在微信主界面上线小范围灰度测试的原生AI助手‘小微’，支持文字/语音交互操控微信原生功能，融合腾讯自研及优质开源多模型技术栈。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-20 02:12</t>
+          <t>2026-06-22 02:40</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-21 02:35</t>
+          <t>2026-06-23 02:05</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -631,14 +631,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HappyOyster 1.0</t>
+          <t>Kimi-Max v2026.06</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>阿里巴巴/通义</t>
+          <t>月之暗面</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -650,29 +650,25 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>交互式世界模型</t>
+          <t>多模态大语言模型</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://www.happyoyster.cn</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>面向交互式内容生成的世界模型，支持动态环境建模与多轮具身交互推演</t>
+          <t>月之暗面发布Kimi-Max新版本，集成实时视频理解、高精度文档解析与跨模态推理能力，专为专业办公与科研场景优化，已接入部分企业API平台。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-20 02:12</t>
+          <t>2026-06-22 02:40</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -687,7 +683,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-06-21 02:35</t>
+          <t>2026-06-23 02:05</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -695,26 +691,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Spark</t>
+          <t>混元T3-Agent</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Google/DeepMind</t>
+          <t>腾讯</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>个人智能体</t>
+          <t>智能体框架</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -722,17 +718,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>谷歌I/O发布的全天候主动式个人智能体，重构搜索引擎从被动查询到主动服务范式</t>
+          <t>腾讯混元团队发布轻量化智能体运行时框架T3-Agent，支持低延迟本地化部署、多工具自动编排与微信生态深度协同，面向小程序与企业服务场景开放内测。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-20 02:12</t>
+          <t>2026-06-22 02:40</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -747,462 +743,10 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-06-21 02:35</t>
+          <t>2026-06-23 02:05</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>&gt;&lt;former (v1.0)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>MIT &amp; MIT-IBM Watson AI Lab</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>neural network architecture</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>一种颠覆性‘中间瘦两头胖’结构的新型Transformer变体，挑战传统等宽层设计，旨在提升能效比与推理效率。</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-06-21 02:36</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Vera CPU (first-generation)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NVIDIA</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>AI-optimized CPU</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-announces-next-generation-ai-platform-rubin-vera-and-nvlink-6</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>英伟达首款独立CPU产品线，专为AI智能体时代token级低延迟调度与多智能体协同推理设计，已交付OpenAI和Anthropic首批试用。</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-06-21 02:36</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Mythos (unreleased public version, but newly designated as 'Frontier Model' under US executive order)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>frontier multimodal LLM</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>虽未正式对外发布新版本，但特朗普6月2日签署行政令明确将Anthropic Mythos列为首批纳入联邦高风险模型评估体系的‘前沿模型’，标志其完成内部迭代并进入监管认定阶段。</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-06-21 02:36</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>OpenAI Personal AGI Assistant (v0.1 prototype)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>智能体（Personal AGI Assistant）</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>OpenAI发布首个面向个人用户的AGI助手原型愿景，聚焦于日常任务、工作、学习与探索的高能力自主智能体，非开源模型，处于内部研究加速阶段规划中。</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-06-22 02:40</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>微信小微（测试版）</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>腾讯</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>原生AI智能体</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>腾讯在微信主界面上线小范围灰度测试的原生AI助手‘小微’，支持文字/语音交互操控微信原生功能，融合腾讯自研及优质开源多模型技术栈。</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-06-22 02:40</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>GLM-5.2</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>智谱AI</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>大语言模型</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>智谱AI正式开源GLM-5.2，为GLM-5系列最新迭代版本，强化长上下文理解、工具调用与多步推理能力，支持1M tokens上下文与结构化输出。</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2026-06-22 02:40</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Kimi-Max v2026.06</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>月之暗面</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>多模态大语言模型</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>月之暗面发布Kimi-Max新版本，集成实时视频理解、高精度文档解析与跨模态推理能力，专为专业办公与科研场景优化，已接入部分企业API平台。</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-06-22 02:40</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>混元T3-Agent</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>腾讯</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>智能体框架</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>腾讯混元团队发布轻量化智能体运行时框架T3-Agent，支持低延迟本地化部署、多工具自动编排与微信生态深度协同，面向小程序与企业服务场景开放内测。</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>2026-06-22 02:40</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-24
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -655,7 +655,11 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://kimi.moonshot.cn/</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>月之暗面发布Kimi-Max新版本，集成实时视频理解、高精度文档解析与跨模态推理能力，专为专业办公与科研场景优化，已接入部分企业API平台。</t>
@@ -747,6 +751,174 @@
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Stellaris-VL 0.8B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>极视角</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>视觉语言大模型（端侧轻量多模态）</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>面向端侧与嵌入式设备的0.8B参数星际视觉语言大模型，支持高性能实时多模态理解与生成。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:08</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>UnisonMind</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>一念科技（清华团队）</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>具身智能体/实时多模态世界模型</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>首个支持流式推理、全模态输入输出、端侧部署的统一具身智能大脑，已实机部署于机器狗、轮椅及服务机器人并完成复杂长程任务验证。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:08</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fugu Ultra</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sakana</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>多智能体编排系统（非单体模型，但属新型AI智能体架构）</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>面向大模型访问中断场景设计的开源多智能体调度与编排系统，支持跨供应商模型路由、动态负载均衡与任务分解，解决前沿模型可用性瓶颈。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:08</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>待核实（LLM交叉巡检发现）</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-25
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OpenAI Personal AGI Assistant (v0.1 prototype)</t>
+          <t>Stellaris-VL 0.8B</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>极视角</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -530,7 +530,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>智能体（Personal AGI Assistant）</t>
+          <t>视觉语言大模型（端侧轻量多模态）</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -538,17 +538,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>OpenAI发布首个面向个人用户的AGI助手原型愿景，聚焦于日常任务、工作、学习与探索的高能力自主智能体，非开源模型，处于内部研究加速阶段规划中。</t>
+          <t>面向端侧与嵌入式设备的0.8B参数星际视觉语言大模型，支持高性能实时多模态理解与生成。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-22 02:40</t>
+          <t>2026-06-24 02:08</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-23 02:05</t>
+          <t>2026-06-25 02:07</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -571,26 +571,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>微信小微（测试版）</t>
+          <t>UnisonMind</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>腾讯</t>
+          <t>一念科技（清华团队）</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>原生AI智能体</t>
+          <t>具身智能体/实时多模态世界模型</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -598,17 +598,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>腾讯在微信主界面上线小范围灰度测试的原生AI助手‘小微’，支持文字/语音交互操控微信原生功能，融合腾讯自研及优质开源多模型技术栈。</t>
+          <t>首个支持流式推理、全模态输入输出、端侧部署的统一具身智能大脑，已实机部署于机器狗、轮椅及服务机器人并完成复杂长程任务验证。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-22 02:40</t>
+          <t>2026-06-24 02:08</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-23 02:05</t>
+          <t>2026-06-25 02:07</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -631,48 +631,48 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kimi-Max v2026.06</t>
+          <t>Fugu Ultra</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>月之暗面</t>
+          <t>Sakana</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>多模态大语言模型</t>
+          <t>多智能体编排系统（非单体模型，但属新型AI智能体架构）</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://kimi.moonshot.cn/</t>
+          <t>https://sakana.ai/fugu</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>月之暗面发布Kimi-Max新版本，集成实时视频理解、高精度文档解析与跨模态推理能力，专为专业办公与科研场景优化，已接入部分企业API平台。</t>
+          <t>面向大模型访问中断场景设计的开源多智能体调度与编排系统，支持跨供应商模型路由、动态负载均衡与任务分解，解决前沿模型可用性瓶颈。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-22 02:40</t>
+          <t>2026-06-24 02:08</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-06-23 02:05</t>
+          <t>2026-06-25 02:07</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -695,26 +695,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>混元T3-Agent</t>
+          <t>鲁班超级智能体（v1.0）</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>腾讯</t>
+          <t>新大陆数字技术</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>智能体框架</t>
+          <t>智能体</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -722,17 +722,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>腾讯混元团队发布轻量化智能体运行时框架T3-Agent，支持低延迟本地化部署、多工具自动编排与微信生态深度协同，面向小程序与企业服务场景开放内测。</t>
+          <t>面向商户全场景经营的AI超级智能体，深度融合Claw互联调度与Hermes智能进化架构，首发36项专属技能，已接入星驿付及慧徕店SaaS体系。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-22 02:40</t>
+          <t>2026-06-25 02:08</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -745,24 +745,20 @@
           <t>待核实（LLM交叉巡检发现）</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-06-23 02:05</t>
-        </is>
-      </c>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Stellaris-VL 0.8B</t>
+          <t>ava数字员工矩阵（含ava me+、avavox、ava app）</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>极视角</t>
+          <t>神州泰岳</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -774,7 +770,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>视觉语言大模型（端侧轻量多模态）</t>
+          <t>智能体/数字员工平台</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -782,17 +778,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>面向端侧与嵌入式设备的0.8B参数星际视觉语言大模型，支持高性能实时多模态理解与生成。</t>
+          <t>在MWC上海正式发布的轻量化企业级数字员工产品矩阵，支持角色化、长期记忆、多Agent协作与统一治理，标志从AI Agent向数字员工范式跃迁。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-06-24 02:08</t>
+          <t>2026-06-25 02:08</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -807,118 +803,6 @@
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>UnisonMind</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>一念科技（清华团队）</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>具身智能体/实时多模态世界模型</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>首个支持流式推理、全模态输入输出、端侧部署的统一具身智能大脑，已实机部署于机器狗、轮椅及服务机器人并完成复杂长程任务验证。</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-06-24 02:08</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Fugu Ultra</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Sakana</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>多智能体编排系统（非单体模型，但属新型AI智能体架构）</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>面向大模型访问中断场景设计的开源多智能体调度与编排系统，支持跨供应商模型路由、动态负载均衡与任务分解，解决前沿模型可用性瓶颈。</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-06-24 02:08</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-27
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,59 +511,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stellaris-VL 0.8B</t>
+          <t>Qwen3-ForcedAligner-0.6B-hf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>极视角</t>
+          <t>阿里</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.6B</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>视觉语言大模型（端侧轻量多模态）</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/Qwen/Qwen3-ForcedAligner-0.6B-hf</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>面向端侧与嵌入式设备的0.8B参数星际视觉语言大模型，支持高性能实时多模态理解与生成。</t>
+          <t>HuggingFace token-classification</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-24 02:08</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Qwen3-ForcedAligner-0.6B-hf)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-25 02:07</t>
+          <t>2026-06-27 02:04</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -571,59 +583,71 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UnisonMind</t>
+          <t>Qwen3-ASR-0.6B-hf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>一念科技（清华团队）</t>
+          <t>阿里</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.6B</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>具身智能体/实时多模态世界模型</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/Qwen/Qwen3-ASR-0.6B-hf</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>首个支持流式推理、全模态输入输出、端侧部署的统一具身智能大脑，已实机部署于机器狗、轮椅及服务机器人并完成复杂长程任务验证。</t>
+          <t>HuggingFace automatic-speech-recognition</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-24 02:08</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Qwen3-ASR-0.6B-hf)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-25 02:07</t>
+          <t>2026-06-27 02:04</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -631,63 +655,71 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fugu Ultra</t>
+          <t>Qwen3-ASR-1.7B-hf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sakana</t>
+          <t>阿里</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1.7B</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>多智能体编排系统（非单体模型，但属新型AI智能体架构）</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://sakana.ai/fugu</t>
+          <t>https://huggingface.co/Qwen/Qwen3-ASR-1.7B-hf</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>面向大模型访问中断场景设计的开源多智能体调度与编排系统，支持跨供应商模型路由、动态负载均衡与任务分解，解决前沿模型可用性瓶颈。</t>
+          <t>HuggingFace automatic-speech-recognition</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-06-24 02:08</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Qwen3-ASR-1.7B-hf)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-06-25 02:07</t>
+          <t>2026-06-27 02:04</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -695,14 +727,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>鲁班超级智能体（v1.0）</t>
+          <t>c-fast-foundationstereo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>新大陆数字技术</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -710,99 +742,55 @@
           <t>国外</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>智能体</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/c-fast-foundationstereo</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>面向商户全场景经营的AI超级智能体，深度融合Claw互联调度与Hermes智能进化架构，首发36项专属技能，已接入星驿付及慧徕店SaaS体系。</t>
+          <t>HuggingFace depth-estimation</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-25 02:08</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/c-fast-foundationstereo)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-06-27 02:04</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ava数字员工矩阵（含ava me+、avavox、ava app）</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>神州泰岳</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>智能体/数字员工平台</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>在MWC上海正式发布的轻量化企业级数字员工产品矩阵，支持角色化、长期记忆、多Agent协作与统一治理，标志从AI Agent向数字员工范式跃迁。</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-06-25 02:08</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>待核实（LLM交叉巡检发现）</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-28
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Qwen3-ForcedAligner-0.6B-hf</t>
+          <t>DeepSeek-V4-Pro-DSpark</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>阿里</t>
+          <t>深度求索</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,11 +531,7 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0.6B</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>基座</t>
@@ -543,39 +539,39 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>non-thinking</t>
+          <t>thinking</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/Qwen/Qwen3-ForcedAligner-0.6B-hf</t>
+          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4-Pro-DSpark</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace token-classification</t>
+          <t>HuggingFace text-generation</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Qwen3-ForcedAligner-0.6B-hf)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/DeepSeek-V4-Pro-DSpark)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-27 02:04</t>
+          <t>2026-06-28 02:15</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -583,14 +579,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Qwen3-ASR-0.6B-hf</t>
+          <t>DeepSeek-V4-Flash-DSpark</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>阿里</t>
+          <t>深度求索</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -603,11 +599,7 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0.6B</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>基座</t>
@@ -615,182 +607,42 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>non-thinking</t>
+          <t>thinking</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/Qwen/Qwen3-ASR-0.6B-hf</t>
+          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4-Flash-DSpark</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace automatic-speech-recognition</t>
+          <t>HuggingFace text-generation</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Qwen3-ASR-0.6B-hf)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/DeepSeek-V4-Flash-DSpark)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-27 02:04</t>
+          <t>2026-06-28 02:15</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Qwen3-ASR-1.7B-hf</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>阿里</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1.7B</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/Qwen/Qwen3-ASR-1.7B-hf</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>HuggingFace automatic-speech-recognition</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(阿里/Qwen3-ASR-1.7B-hf)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-06-27 02:04</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>c-fast-foundationstereo</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/c-fast-foundationstereo</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>HuggingFace depth-estimation</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/c-fast-foundationstereo)</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-06-27 02:04</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-06-29
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DeepSeek-V4-Pro-DSpark</t>
+          <t>eagle3_gemma4_12b_ttt7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -539,39 +539,39 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>thinking</t>
+          <t>non-thinking</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4-Pro-DSpark</t>
+          <t>https://huggingface.co/deepseek-ai/eagle3_gemma4_12b_ttt7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace text-generation</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/DeepSeek-V4-Pro-DSpark)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/eagle3_gemma4_12b_ttt7)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-28 02:15</t>
+          <t>2026-06-29 02:14</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -579,7 +579,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DeepSeek-V4-Flash-DSpark</t>
+          <t>eagle3_qwen3_14b_ttt7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -607,42 +607,722 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>thinking</t>
+          <t>non-thinking</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4-Flash-DSpark</t>
+          <t>https://huggingface.co/deepseek-ai/eagle3_qwen3_14b_ttt7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace text-generation</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/DeepSeek-V4-Flash-DSpark)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/eagle3_qwen3_14b_ttt7)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-28 02:15</t>
+          <t>2026-06-29 02:14</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eagle3_qwen3_8b_ttt7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/eagle3_qwen3_8b_ttt7</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/eagle3_qwen3_8b_ttt7)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>eagle3_qwen3_4b_ttt7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/eagle3_qwen3_4b_ttt7</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/eagle3_qwen3_4b_ttt7)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dflash_gemma4_12b_block7</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dflash_gemma4_12b_block7</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dflash_gemma4_12b_block7)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dflash_qwen3_14b_block7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dflash_qwen3_14b_block7</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dflash_qwen3_14b_block7)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dflash_qwen3_8b_block7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dflash_qwen3_8b_block7</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dflash_qwen3_8b_block7)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dflash_qwen3_4b_block7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dflash_qwen3_4b_block7</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dflash_qwen3_4b_block7)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dspark_gemma4_12b_block7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dspark_gemma4_12b_block7</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dspark_gemma4_12b_block7)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dspark_qwen3_14b_block7</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dspark_qwen3_14b_block7</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dspark_qwen3_14b_block7)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dspark_qwen3_8b_block7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dspark_qwen3_8b_block7</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dspark_qwen3_8b_block7)</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dspark_qwen3_4b_block7</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>深度求索</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/dspark_qwen3_4b_block7</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/dspark_qwen3_4b_block7)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-06-29 02:14</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-03
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5</t>
+          <t>HARC-Qwen2.5-7B-Instruct</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>微软</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,58 +528,54 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>闭源</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>多模态</t>
+          <t>基座</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/claude-sonnet-5</t>
+          <t>https://huggingface.co/microsoft/HARC-Qwen2.5-7B-Instruct</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1000k上下文；顶级编码能力</t>
+          <t>HuggingFace text-generation</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/HARC-Qwen2.5-7B-Instruct)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-01 02:13</t>
+          <t>2026-07-03 01:50</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -587,7 +583,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GELab-Zero-4B-preview-Sico-Evolution</t>
+          <t>HARC-Llama-3.1-8B-Instruct</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -609,12 +605,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4B</t>
+          <t>8B</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>基座</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -625,33 +621,33 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/GELab-Zero-4B-preview-Sico-Evolution</t>
+          <t>https://huggingface.co/microsoft/HARC-Llama-3.1-8B-Instruct</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace image-text-to-text</t>
+          <t>HuggingFace text-generation</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/GELab-Zero-4B-preview-Sico-Evolution)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/HARC-Llama-3.1-8B-Instruct)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-07-01 02:13</t>
+          <t>2026-07-03 01:50</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-06
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HARC-Qwen2.5-7B-Instruct</t>
+          <t>gr00t17-lerobot-libero_goal-640</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,14 +531,10 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>7B</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>基座</t>
+          <t>未知</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -549,33 +545,33 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/HARC-Qwen2.5-7B-Instruct</t>
+          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_goal-640</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace text-generation</t>
+          <t>HuggingFace robotics</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/HARC-Qwen2.5-7B-Instruct)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_goal-640)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-03 01:50</t>
+          <t>2026-07-06 02:02</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -583,14 +579,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HARC-Llama-3.1-8B-Instruct</t>
+          <t>gr00t17-lerobot-libero_10-640</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -603,14 +599,10 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>8B</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>基座</t>
+          <t>未知</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -621,36 +613,172 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/HARC-Llama-3.1-8B-Instruct</t>
+          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_10-640</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace text-generation</t>
+          <t>HuggingFace robotics</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/HARC-Llama-3.1-8B-Instruct)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_10-640)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-07-03 01:50</t>
+          <t>2026-07-06 02:02</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>gr00t17-lerobot-libero_object-640</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_object-640</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HuggingFace robotics</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_object-640)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-07-06 02:02</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>gr00t17-lerobot-libero_spatial-640</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_spatial-640</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>HuggingFace robotics</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_spatial-640)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-07-06 02:02</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-08
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>gr00t17-lerobot-libero_goal-640</t>
+          <t>CWIP-1.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -545,240 +545,36 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_goal-640</t>
+          <t>https://huggingface.co/nvidia/CWIP-1.0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace robotics</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_goal-640)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/CWIP-1.0)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-06 02:02</t>
+          <t>2026-07-08 01:27</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>gr00t17-lerobot-libero_10-640</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_10-640</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>HuggingFace robotics</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_10-640)</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-07-06 02:02</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>gr00t17-lerobot-libero_object-640</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_object-640</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>HuggingFace robotics</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_object-640)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-07-06 02:02</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>gr00t17-lerobot-libero_spatial-640</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/gr00t17-lerobot-libero_spatial-640</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>HuggingFace robotics</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/gr00t17-lerobot-libero_spatial-640)</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-07-06 02:02</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-09
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CWIP-1.0</t>
+          <t>nvDock</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -545,7 +545,7 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/CWIP-1.0</t>
+          <t>https://huggingface.co/nvidia/nvDock</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -555,23 +555,23 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/CWIP-1.0)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/nvDock)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-08 01:27</t>
+          <t>2026-07-09 01:49</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-15
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nvDock</t>
+          <t>Nemotron-3-Embed-1B-NVFP4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -531,21 +531,25 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>基座</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>non-thinking</t>
+          <t>thinking</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/nvDock</t>
+          <t>https://huggingface.co/nvidia/Nemotron-3-Embed-1B-NVFP4</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -555,26 +559,170 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/nvDock)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Nemotron-3-Embed-1B-NVFP4)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-09 01:49</t>
+          <t>2026-07-15 01:16</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nemotron-3-Embed-8B-BF16</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8B</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/Nemotron-3-Embed-8B-BF16</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>HuggingFace sentence-similarity</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Nemotron-3-Embed-8B-BF16)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-07-15 01:16</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nemotron-3-Embed-1B-BF16</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/Nemotron-3-Embed-1B-BF16</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HuggingFace sentence-similarity</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Nemotron-3-Embed-1B-BF16)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-07-15 01:16</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-16
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nemotron-3-Embed-1B-NVFP4</t>
+          <t>bitnet-embedding-0.6b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>微软</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -533,23 +533,23 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>0.6B</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>基座</t>
+          <t>未知</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>thinking</t>
+          <t>non-thinking</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/Nemotron-3-Embed-1B-NVFP4</t>
+          <t>https://huggingface.co/microsoft/bitnet-embedding-0.6b</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -559,23 +559,23 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Nemotron-3-Embed-1B-NVFP4)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/bitnet-embedding-0.6b)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-15 01:16</t>
+          <t>2026-07-16 01:26</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -583,14 +583,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nemotron-3-Embed-8B-BF16</t>
+          <t>bitnet-embedding-270m</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>微软</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -605,124 +605,52 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>270M</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>基座</t>
+          <t>未知</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>thinking</t>
+          <t>non-thinking</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/Nemotron-3-Embed-8B-BF16</t>
+          <t>https://huggingface.co/microsoft/bitnet-embedding-270m</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace sentence-similarity</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Nemotron-3-Embed-8B-BF16)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/bitnet-embedding-270m)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-07-15 01:16</t>
+          <t>2026-07-16 01:26</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Nemotron-3-Embed-1B-BF16</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/Nemotron-3-Embed-1B-BF16</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>HuggingFace sentence-similarity</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/Nemotron-3-Embed-1B-BF16)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-07-15 01:16</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-22
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bitnet-embedding-0.6b</t>
+          <t>Gemini 3.5 Flash Cyber</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,17 +528,13 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0.6B</t>
-        </is>
-      </c>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>基座</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -546,36 +542,44 @@
           <t>non-thinking</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/bitnet-embedding-0.6b</t>
+          <t>https://llm-stats.com/models/gemini-3.5-flash-cyber</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>针对网络安全用途；协助发现、验证及修补软件漏洞；仅向政府及受信任合作伙伴开放</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/bitnet-embedding-0.6b)</t>
+          <t>llm-stats.com 排行榜</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-16 01:26</t>
+          <t>2026-07-22 01:25</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -583,14 +587,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bitnet-embedding-270m</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -600,17 +604,13 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>270M</t>
-        </is>
-      </c>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>多模态</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -618,39 +618,123 @@
           <t>non-thinking</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/bitnet-embedding-270m</t>
+          <t>https://llm-stats.com/models/gemini-3.5-flash-lite</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>1048k上下文</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/bitnet-embedding-270m)</t>
+          <t>llm-stats.com 排行榜</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-07-16 01:26</t>
+          <t>2026-07-22 01:25</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Gemini 3.6 Flash</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/gemini-3.6-flash</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1048k上下文</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-07-22 01:25</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-25
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash Cyber</t>
+          <t>Claude Opus 5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -534,12 +534,12 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>基座</t>
+          <t>多模态</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>non-thinking</t>
+          <t>thinking</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -549,22 +549,22 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/gemini-3.5-flash-cyber</t>
+          <t>https://llm-stats.com/models/claude-opus-5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>针对网络安全用途；协助发现、验证及修补软件漏洞；仅向政府及受信任合作伙伴开放</t>
+          <t>1000k上下文；高端定价</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-22 01:25</t>
+          <t>2026-07-25 01:29</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -587,14 +587,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>VibeVoice-ASR-BitNet</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>微软</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -604,13 +604,13 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>闭源</t>
+          <t>开源</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>多模态</t>
+          <t>语音</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -618,123 +618,39 @@
           <t>non-thinking</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/gemini-3.5-flash-lite</t>
+          <t>https://huggingface.co/microsoft/VibeVoice-ASR-BitNet</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1048k上下文</t>
+          <t>HuggingFace automatic-speech-recognition</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/VibeVoice-ASR-BitNet)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-07-22 01:25</t>
+          <t>2026-07-25 01:29</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Gemini 3.6 Flash</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>多模态</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1048k上下文</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>llm-stats.com 排行榜</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-07-22 01:25</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-27
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Claude Opus 5</t>
+          <t>Mage-ViT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>微软</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,129 +528,53 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>闭源</t>
+          <t>开源</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>多模态</t>
+          <t>未知</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/claude-opus-5</t>
+          <t>https://huggingface.co/microsoft/Mage-ViT</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1000k上下文；高端定价</t>
+          <t>HuggingFace image-feature-extraction</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(微软/Mage-ViT)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-25 01:29</t>
+          <t>2026-07-27 01:50</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>VibeVoice-ASR-BitNet</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>微软</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>语音</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/microsoft/VibeVoice-ASR-BitNet</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>HuggingFace automatic-speech-recognition</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/VibeVoice-ASR-BitNet)</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-07-25 01:29</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-07-31
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mage-ViT</t>
+          <t>K-EXAONE-2.0-750B-A37B-DSpark</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>微软</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,7 +531,11 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>750B(A37B)</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>未知</t>
@@ -545,36 +549,180 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/microsoft/Mage-ViT</t>
+          <t>https://huggingface.co/LGAI-EXAONE/K-EXAONE-2.0-750B-A37B-DSpark</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace image-feature-extraction</t>
+          <t>HuggingFace text-generation</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(微软/Mage-ViT)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(lg/K-EXAONE-2.0-750B-A37B-DSpark)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-27 01:50</t>
+          <t>2026-07-31 01:45</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>K-EXAONE-2.0-750B-A37B-NVFP4</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LG</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>750B(A37B)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/LGAI-EXAONE/K-EXAONE-2.0-750B-A37B-NVFP4</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(lg/K-EXAONE-2.0-750B-A37B-NVFP4)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-07-31 01:45</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>K-EXAONE-2.0-750B-A37B-FP8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LG</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>750B(A37B)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/LGAI-EXAONE/K-EXAONE-2.0-750B-A37B-FP8</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(lg/K-EXAONE-2.0-750B-A37B-FP8)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-07-31 01:45</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-08-01
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,19 +511,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>K-EXAONE-2.0-750B-A37B-DSpark</t>
+          <t>DeepSeek-V4-Flash-0731</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>深度求索</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -531,25 +531,21 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>750B(A37B)</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>基座</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>non-thinking</t>
+          <t>thinking</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/LGAI-EXAONE/K-EXAONE-2.0-750B-A37B-DSpark</t>
+          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4-Flash-0731</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -559,170 +555,26 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(lg/K-EXAONE-2.0-750B-A37B-DSpark)</t>
+          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/DeepSeek-V4-Flash-0731)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-31 01:45</t>
+          <t>2026-08-01 01:46</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>K-EXAONE-2.0-750B-A37B-NVFP4</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LG</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>750B(A37B)</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/LGAI-EXAONE/K-EXAONE-2.0-750B-A37B-NVFP4</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(lg/K-EXAONE-2.0-750B-A37B-NVFP4)</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-07-31 01:45</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>K-EXAONE-2.0-750B-A37B-FP8</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LG</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>750B(A37B)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>non-thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/LGAI-EXAONE/K-EXAONE-2.0-750B-A37B-FP8</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(lg/K-EXAONE-2.0-750B-A37B-FP8)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-07-31 01:45</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-08-12
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -511,19 +511,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DeepSeek-V4-Flash-0731</t>
+          <t>Nemotron 3.5 Lightning (30B A3B)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>深度求索</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国内</t>
+          <t>国外</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -531,7 +531,11 @@
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>基座</t>
@@ -542,36 +546,44 @@
           <t>thinking</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4-Flash-0731</t>
+          <t>https://llm-stats.com/models/nemotron-3.5-lightning-30b-a3b</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HuggingFace text-generation</t>
+          <t>MoE架构；30B参数；262k上下文；低成本；Openmdw</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(深度求索/DeepSeek-V4-Flash-0731)</t>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(nvidia/Nemotron 3.5 Lightning (30B A3B))</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-08-01 01:46</t>
+          <t>2026-08-12 00:58</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-08-13
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nemotron 3.5 Lightning (30B A3B)</t>
+          <t>Grok 4.6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>xAI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,65 +528,141 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/grok-4.6</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>500k上下文</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2026-08-13 01:00</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LFM2.5-VL-3B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Liquid AI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>开源</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>30B</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>non-thinking</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>通用对话</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/nemotron-3.5-lightning-30b-a3b</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>MoE架构；30B参数；262k上下文；低成本；Openmdw</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/lfm-2.5-vl-3b</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Lfm1 0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>llm-stats.com 排行榜 · HuggingFace 需登录(nvidia/Nemotron 3.5 Lightning (30B A3B))</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2026-08-12 00:58</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(liquid-ai/LFM2.5-VL-3B)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-08-13 01:00</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-08-14
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -511,30 +511,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Grok 4.6</t>
+          <t>DeepSeek-V4-Pro-0813</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>国外</t>
+          <t>国内</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>闭源</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2T</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>多模态</t>
+          <t>基座</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -549,22 +553,22 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/grok-4.6</t>
+          <t>https://llm-stats.com/models/deepseek-v4-pro-0813</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>500k上下文</t>
+          <t>MoE架构；2T参数；1048k上下文；MIT</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -574,12 +578,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜</t>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(deepseek/DeepSeek-V4-Pro-0813)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-08-13 01:00</t>
+          <t>2026-08-14 00:59</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -587,14 +591,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LFM2.5-VL-3B</t>
+          <t>Gemini 3.7 Flash</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Liquid AI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -604,14 +608,10 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>多模态</t>
@@ -619,7 +619,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>non-thinking</t>
+          <t>thinking</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -629,22 +629,22 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/lfm-2.5-vl-3b</t>
+          <t>https://llm-stats.com/models/gemini-3.7-flash</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Lfm1 0</t>
+          <t>1048k上下文</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -654,12 +654,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜 · HuggingFace 需登录(liquid-ai/LFM2.5-VL-3B)</t>
+          <t>llm-stats.com 排行榜</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-08-13 01:00</t>
+          <t>2026-08-14 00:59</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-08-15
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DeepSeek-V4-Pro-0813</t>
+          <t>Qwen3.8-27B</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Alibaba Cloud / Qwen Team</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -533,12 +533,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2T</t>
+          <t>28B</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>基座</t>
+          <t>多模态</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -553,22 +553,22 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/deepseek-v4-pro-0813</t>
+          <t>https://llm-stats.com/models/qwen3.8-27b</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>MoE架构；2T参数；1048k上下文；MIT</t>
+          <t>强推理能力；Apache 2.0</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -578,12 +578,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜 · HuggingFace 需登录(deepseek/DeepSeek-V4-Pro-0813)</t>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(alibaba-cloud-/Qwen3.8-27B)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-08-14 00:59</t>
+          <t>2026-08-15 00:34</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -591,78 +591,422 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gemini 3.7 Flash</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Zhipu AI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>753B</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/glm-5.3</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>MoE架构；753B参数；Unknown</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-08-15 00:34</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NVIDIA-Nemotron-Labs-Teacher-Chat</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>国外</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>多模态</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>thinking</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/gemini-3.7-flash</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1048k上下文</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-Chat</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>llm-stats.com 排行榜</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-08-14 00:59</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-Chat)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-08-15 00:34</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NVIDIA-Nemotron-Labs-Teacher-Competition-Coding</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-Competition-Coding</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-Competition-Coding)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-08-15 00:34</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NVIDIA-Nemotron-Labs-Teacher-Instruction-Following</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-Instruction-Following</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-Instruction-Following)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-08-15 00:34</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NVIDIA-Nemotron-Labs-Teacher-General-Reasoning</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-General-Reasoning</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-General-Reasoning)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-08-15 00:34</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NVIDIA-Nemotron-Labs-Teacher-STEM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>英伟达</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>基座</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-STEM</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>HuggingFace text-generation</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-STEM)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-08-15 00:34</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auto): daily pipeline 2026-08-22
</commit_message>
<xml_diff>
--- a/Model_Navigate/data/Object-Models-Updated.xlsx
+++ b/Model_Navigate/data/Object-Models-Updated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,14 +511,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Qwen3.8-27B</t>
+          <t>DeepSeek-V4-Flash-Vision-Exp</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Alibaba Cloud / Qwen Team</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,14 +528,10 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>28B</t>
-        </is>
-      </c>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>多模态</t>
@@ -553,22 +549,22 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://llm-stats.com/models/qwen3.8-27b</t>
+          <t>https://llm-stats.com/models/deepseek-v4-flash-vision-exp</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>强推理能力；Apache 2.0</t>
+          <t>1048k上下文；低成本；Unknown</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -578,435 +574,15 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>llm-stats.com 排行榜 · HuggingFace 需登录(alibaba-cloud-/Qwen3.8-27B)</t>
+          <t>llm-stats.com 排行榜</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-08-15 00:34</t>
+          <t>2026-08-22 00:34</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>GLM-5.3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Zhipu AI</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>国内</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>闭源</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>753B</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>通用对话</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://llm-stats.com/models/glm-5.3</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>MoE架构；753B参数；Unknown</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>llm-stats.com 排行榜</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-08-15 00:34</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>NVIDIA-Nemotron-Labs-Teacher-Chat</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-Chat</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-Chat)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-08-15 00:34</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NVIDIA-Nemotron-Labs-Teacher-Competition-Coding</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-Competition-Coding</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-Competition-Coding)</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-08-15 00:34</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>NVIDIA-Nemotron-Labs-Teacher-Instruction-Following</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-Instruction-Following</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-Instruction-Following)</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-08-15 00:34</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>NVIDIA-Nemotron-Labs-Teacher-General-Reasoning</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-General-Reasoning</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-General-Reasoning)</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>2026-08-15 00:34</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>NVIDIA-Nemotron-Labs-Teacher-STEM</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>英伟达</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>国外</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>开源</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>基座</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/nvidia/NVIDIA-Nemotron-Labs-Teacher-STEM</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>HuggingFace text-generation</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · HuggingFace 需登录(英伟达/NVIDIA-Nemotron-Labs-Teacher-STEM)</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>2026-08-15 00:34</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>